<commit_message>
docs: add more verified QNN and QRNN papers
</commit_message>
<xml_diff>
--- a/metadata/QNN-QRNN.xlsx
+++ b/metadata/QNN-QRNN.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rd37a9d763f7b429b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R562438961026421f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -1948,19 +1948,19 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9" s="2" t="str">
-        <x:v>Quantum Gated Recurrent Neural Networks</x:v>
+        <x:v>Lightweight quantum recurrent neural networks for time-series and dynamical systems</x:v>
       </x:c>
       <x:c r="B9" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C9" s="2" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D9" s="2" t="str">
-        <x:v>Yanan Li; Zhimin Wang; Ruipeng Xing; Shao Changheng; Shangshang Shi; Jiaxin Li; Guoqiang Zhong; Yongjian Gu</x:v>
+        <x:v>Yuan Chen; Abdul Khaliq</x:v>
       </x:c>
       <x:c r="E9" s="2" t="str">
-        <x:v>https://doi.org/10.1109/TPAMI.2024.3519605</x:v>
+        <x:v>https://doi.org/10.1016/j.asoc.2026.114949</x:v>
       </x:c>
       <x:c r="F9" s="2" t="str">
         <x:v>QRNN</x:v>
@@ -1968,39 +1968,39 @@
     </x:row>
     <x:row r="10">
       <x:c r="A10" s="2" t="str">
-        <x:v>HQRNN-FD: A Hybrid Quantum Recurrent Neural Network for Fraud Detection</x:v>
+        <x:v>CQNAS: Convolutional quantum hybrid neural network architecture search for image classification</x:v>
       </x:c>
       <x:c r="B10" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C10" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D10" s="2" t="str">
-        <x:v>Yao-Chong Li; Yi-Fan Zhang; Rui-Qing Xu; Ri-Gui Zhou; Yi-Lin Dong</x:v>
+        <x:v>Desheng Kong; Jiaying Jin; Xiangshuo Cui; J. Yan; J. Tang; Yulong Fu; Jing Xu; Donglin Wang</x:v>
       </x:c>
       <x:c r="E10" s="2" t="str">
-        <x:v>https://doi.org/10.3390/e27090906</x:v>
+        <x:v>https://doi.org/10.1016/j.neucom.2026.133236</x:v>
       </x:c>
       <x:c r="F10" s="2" t="str">
-        <x:v>QRNN</x:v>
+        <x:v>QNN</x:v>
       </x:c>
     </x:row>
     <x:row r="11">
       <x:c r="A11" s="2" t="str">
-        <x:v>Exploring Quantum Neural Networks for Demand Forecasting</x:v>
+        <x:v>Quantum Fourier Transform Neural Network with image blockwise representation for image classification</x:v>
       </x:c>
       <x:c r="B11" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C11" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D11" s="2" t="str">
-        <x:v>Gleydson Fernandes de Jesus; Maria Heloísa Fraga da Silva; Otto Menegasso Pires; Lucas Cruz da Silva; Clebson Dos Santos Cruz; Valéria Loureiro da Silva</x:v>
+        <x:v>Desheng Kong; Kangning An; Kairan Zhang; Mingyang Yu; Yulong Fu; Wei Wang; Jing Xu; Donglin Wang</x:v>
       </x:c>
       <x:c r="E11" s="2" t="str">
-        <x:v>https://doi.org/10.3390/e27050490</x:v>
+        <x:v>https://doi.org/10.1016/j.knosys.2026.115937</x:v>
       </x:c>
       <x:c r="F11" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2008,19 +2008,19 @@
     </x:row>
     <x:row r="12" ht="15.75" customHeight="1">
       <x:c r="A12" s="3" t="str">
-        <x:v>Quantum neural networks with data re-uploading for urban traffic time series forecasting</x:v>
+        <x:v>Quantum computational sensing using quantum signal processing, quantum neural networks, and Hamiltonian engineering</x:v>
       </x:c>
       <x:c r="B12" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C12" s="2" t="str">
         <x:v>Springer Nature</x:v>
       </x:c>
       <x:c r="D12" s="2" t="str">
-        <x:v>Nikolaos Schetakis; Paolo Bonfini; Negin Alisoltani; Konstantinos Blazakis; Symeon I. Tsintzos; Alexis Askitopoulos; Davit Aghamalyan; Panagiotis Fafoutellis; Eleni I. Vlahogianni</x:v>
+        <x:v>Saeed A. Khan; Sridhar Prabhu; Logan G. Wright; Peter L. McMahon</x:v>
       </x:c>
       <x:c r="E12" s="2" t="str">
-        <x:v>https://doi.org/10.1038/s41598-025-04546-8</x:v>
+        <x:v>https://doi.org/10.1038/s41534-026-01235-w</x:v>
       </x:c>
       <x:c r="F12" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2028,19 +2028,19 @@
     </x:row>
     <x:row r="13">
       <x:c r="A13" s="2" t="str">
-        <x:v>A Quantum Spatial Graph Convolutional Neural Network Model on Quantum Circuits</x:v>
+        <x:v>Quantum convolutional neural network for MRI brain tumor analysis: Binary and multiclass classification using a four-qubit architecture</x:v>
       </x:c>
       <x:c r="B13" s="2" t="n">
-        <x:v>2025</x:v>
+        <x:v>2026</x:v>
       </x:c>
       <x:c r="C13" s="2" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D13" s="2" t="str">
-        <x:v>Jin Zheng; Qing Gao; Maciej Ogorzalek; Jinhu Lu; Yue Deng</x:v>
+        <x:v>Sitti Yani; Sugih Pratama Nugraha; Ariiq Islam Alfajri; Tony Sumaryada; Duong Thanh Tai; Hiba Omer; Nissren Tamam; Abdelmoneim Sulieman</x:v>
       </x:c>
       <x:c r="E13" s="2" t="str">
-        <x:v>https://doi.org/10.1109/TNNLS.2024.3382174</x:v>
+        <x:v>https://doi.org/10.1016/j.radphyschem.2025.113545</x:v>
       </x:c>
       <x:c r="F13" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2048,7 +2048,7 @@
     </x:row>
     <x:row r="14">
       <x:c r="A14" s="2" t="str">
-        <x:v>NR-QNN: Noise-Resilient Quantum Neural Network</x:v>
+        <x:v>Quantum Gated Recurrent Neural Networks</x:v>
       </x:c>
       <x:c r="B14" s="2" t="n">
         <x:v>2025</x:v>
@@ -2057,151 +2057,151 @@
         <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D14" s="2" t="str">
-        <x:v>Sohrab Sajadimanesh; Hanieh Aghaee Rad; Jean Paul Latyr Faye; Ehsan Atoofian</x:v>
+        <x:v>Yanan Li; Zhimin Wang; Ruipeng Xing; Shao Changheng; Shangshang Shi; Jiaxin Li; Guoqiang Zhong; Yongjian Gu</x:v>
       </x:c>
       <x:c r="E14" s="2" t="str">
-        <x:v>https://doi.org/10.1109/ACCESS.2025.3546956</x:v>
+        <x:v>https://doi.org/10.1109/TPAMI.2024.3519605</x:v>
       </x:c>
       <x:c r="F14" s="2" t="str">
-        <x:v>QNN</x:v>
+        <x:v>QRNN</x:v>
       </x:c>
     </x:row>
     <x:row r="15">
       <x:c r="A15" s="2" t="str">
+        <x:v>HQRNN-FD: A Hybrid Quantum Recurrent Neural Network for Fraud Detection</x:v>
+      </x:c>
+      <x:c r="B15" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C15" s="2" t="str">
+        <x:v>MDPI</x:v>
+      </x:c>
+      <x:c r="D15" s="2" t="str">
+        <x:v>Yao-Chong Li; Yi-Fan Zhang; Rui-Qing Xu; Ri-Gui Zhou; Yi-Lin Dong</x:v>
+      </x:c>
+      <x:c r="E15" s="2" t="str">
+        <x:v>https://doi.org/10.3390/e27090906</x:v>
+      </x:c>
+      <x:c r="F15" s="2" t="str">
+        <x:v>QRNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" s="2" t="str">
+        <x:v>Exploring Quantum Neural Networks for Demand Forecasting</x:v>
+      </x:c>
+      <x:c r="B16" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C16" s="2" t="str">
+        <x:v>MDPI</x:v>
+      </x:c>
+      <x:c r="D16" s="2" t="str">
+        <x:v>Gleydson Fernandes de Jesus; Maria Heloísa Fraga da Silva; Otto Menegasso Pires; Lucas Cruz da Silva; Clebson Dos Santos Cruz; Valéria Loureiro da Silva</x:v>
+      </x:c>
+      <x:c r="E16" s="2" t="str">
+        <x:v>https://doi.org/10.3390/e27050490</x:v>
+      </x:c>
+      <x:c r="F16" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="17">
+      <x:c r="A17" s="2" t="str">
+        <x:v>Quantum neural networks with data re-uploading for urban traffic time series forecasting</x:v>
+      </x:c>
+      <x:c r="B17" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C17" s="2" t="str">
+        <x:v>Springer Nature</x:v>
+      </x:c>
+      <x:c r="D17" s="2" t="str">
+        <x:v>Nikolaos Schetakis; Paolo Bonfini; Negin Alisoltani; Konstantinos Blazakis; Symeon I. Tsintzos; Alexis Askitopoulos; Davit Aghamalyan; Panagiotis Fafoutellis; Eleni I. Vlahogianni</x:v>
+      </x:c>
+      <x:c r="E17" s="2" t="str">
+        <x:v>https://doi.org/10.1038/s41598-025-04546-8</x:v>
+      </x:c>
+      <x:c r="F17" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="18">
+      <x:c r="A18" s="2" t="str">
+        <x:v>A Quantum Spatial Graph Convolutional Neural Network Model on Quantum Circuits</x:v>
+      </x:c>
+      <x:c r="B18" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C18" s="2" t="str">
+        <x:v>IEEE</x:v>
+      </x:c>
+      <x:c r="D18" s="2" t="str">
+        <x:v>Jin Zheng; Qing Gao; Maciej Ogorzalek; Jinhu Lu; Yue Deng</x:v>
+      </x:c>
+      <x:c r="E18" s="2" t="str">
+        <x:v>https://doi.org/10.1109/TNNLS.2024.3382174</x:v>
+      </x:c>
+      <x:c r="F18" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="19">
+      <x:c r="A19" s="2" t="str">
+        <x:v>NR-QNN: Noise-Resilient Quantum Neural Network</x:v>
+      </x:c>
+      <x:c r="B19" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C19" s="2" t="str">
+        <x:v>IEEE</x:v>
+      </x:c>
+      <x:c r="D19" s="2" t="str">
+        <x:v>Sohrab Sajadimanesh; Hanieh Aghaee Rad; Jean Paul Latyr Faye; Ehsan Atoofian</x:v>
+      </x:c>
+      <x:c r="E19" s="2" t="str">
+        <x:v>https://doi.org/10.1109/ACCESS.2025.3546956</x:v>
+      </x:c>
+      <x:c r="F19" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="20">
+      <x:c r="A20" s="2" t="str">
+        <x:v>Quantum neural networks form Gaussian processes</x:v>
+      </x:c>
+      <x:c r="B20" s="2" t="n">
+        <x:v>2025</x:v>
+      </x:c>
+      <x:c r="C20" s="2" t="str">
+        <x:v>Nature Physics</x:v>
+      </x:c>
+      <x:c r="D20" s="2" t="str">
+        <x:v>Diego García-Martín; Martín Larocca; M. Cerezo</x:v>
+      </x:c>
+      <x:c r="E20" s="2" t="str">
+        <x:v>https://doi.org/10.1038/s41567-025-02883-z</x:v>
+      </x:c>
+      <x:c r="F20" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="21">
+      <x:c r="A21" s="2" t="str">
         <x:v>QuanTest: Entanglement-Guided Testing of Quantum Neural Network Systems
 </x:v>
       </x:c>
-      <x:c r="B15" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C15" s="2" t="str">
-        <x:v>ACM Transactions on Software Engineering and Methodology</x:v>
-      </x:c>
-      <x:c r="D15" s="2" t="str">
-        <x:v>Shi, Jinjing</x:v>
-      </x:c>
-      <x:c r="E15" s="2" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3688840</x:v>
-      </x:c>
-      <x:c r="F15" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="16">
-      <x:c r="A16" s="2" t="str">
-        <x:v>Application of Quantum Neural Network for Solar Irradiance Forecasting: A Case Study Using the Folsom Dataset, California</x:v>
-      </x:c>
-      <x:c r="B16" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C16" s="2" t="str">
-        <x:v>Energies</x:v>
-      </x:c>
-      <x:c r="D16" s="2" t="str">
-        <x:v>Oliveira Santos, Victor, </x:v>
-      </x:c>
-      <x:c r="E16" s="2" t="str">
-        <x:v>https://www.mdpi.com/1996-1073/17/14/3580</x:v>
-      </x:c>
-      <x:c r="F16" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="17">
-      <x:c r="A17" s="2" t="str">
-        <x:v>hybrid quantum neural network structures for image multi-classification</x:v>
-      </x:c>
-      <x:c r="B17" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C17" s="2" t="str">
-        <x:v>Physica Scripta </x:v>
-      </x:c>
-      <x:c r="D17" s="2" t="str">
-        <x:v>Shi, Mingrui, Haozhen Situ,</x:v>
-      </x:c>
-      <x:c r="E17" s="2" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/1402-4896/ad3e3d/meta</x:v>
-      </x:c>
-      <x:c r="F17" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="18">
-      <x:c r="A18" s="2" t="str">
-        <x:v>Optimization enabled Deep Quantum Neural Network for weed classification and density estimation</x:v>
-      </x:c>
-      <x:c r="B18" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C18" s="2" t="str">
-        <x:v>Expert Systems with Applications </x:v>
-      </x:c>
-      <x:c r="D18" s="2" t="str">
-        <x:v>Veeragandham, Syamasudha,</x:v>
-      </x:c>
-      <x:c r="E18" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0957417423031810</x:v>
-      </x:c>
-      <x:c r="F18" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="19">
-      <x:c r="A19" s="2" t="str">
-        <x:v>Estimating quantum mutual information through a quantum neural network</x:v>
-      </x:c>
-      <x:c r="B19" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C19" s="2" t="str">
-        <x:v>Quantum Information Processing</x:v>
-      </x:c>
-      <x:c r="D19" s="2" t="str">
-        <x:v>Shin, Myeongjin</x:v>
-      </x:c>
-      <x:c r="E19" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11128-023-04253-1</x:v>
-      </x:c>
-      <x:c r="F19" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="20">
-      <x:c r="A20" s="2" t="str">
-        <x:v>Superposition-enhanced quantum neural network for multi-class image classification</x:v>
-      </x:c>
-      <x:c r="B20" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C20" s="2" t="str">
-        <x:v>Journal of Physics </x:v>
-      </x:c>
-      <x:c r="D20" s="2" t="str">
-        <x:v>Bai, Qi, and Xianliang</x:v>
-      </x:c>
-      <x:c r="E20" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0577907324001151</x:v>
-      </x:c>
-      <x:c r="F20" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="21">
-      <x:c r="A21" s="2" t="str">
-        <x:v>Restricting to the chip architecture maintains the quantum neural network accuracy</x:v>
-      </x:c>
       <x:c r="B21" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C21" s="2" t="str">
-        <x:v>Quantum Information Processing</x:v>
+        <x:v>ACM Transactions on Software Engineering and Methodology</x:v>
       </x:c>
       <x:c r="D21" s="2" t="str">
-        <x:v>Friedrich, Lucas,</x:v>
+        <x:v>Shi, Jinjing</x:v>
       </x:c>
       <x:c r="E21" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11128-024-04336-7</x:v>
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3688840</x:v>
       </x:c>
       <x:c r="F21" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2209,222 +2209,222 @@
     </x:row>
     <x:row r="22">
       <x:c r="A22" s="2" t="str">
+        <x:v>Application of Quantum Neural Network for Solar Irradiance Forecasting: A Case Study Using the Folsom Dataset, California</x:v>
+      </x:c>
+      <x:c r="B22" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C22" s="2" t="str">
+        <x:v>Energies</x:v>
+      </x:c>
+      <x:c r="D22" s="2" t="str">
+        <x:v>Oliveira Santos, Victor, </x:v>
+      </x:c>
+      <x:c r="E22" s="2" t="str">
+        <x:v>https://www.mdpi.com/1996-1073/17/14/3580</x:v>
+      </x:c>
+      <x:c r="F22" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="23">
+      <x:c r="A23" s="2" t="str">
+        <x:v>hybrid quantum neural network structures for image multi-classification</x:v>
+      </x:c>
+      <x:c r="B23" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C23" s="2" t="str">
+        <x:v>Physica Scripta </x:v>
+      </x:c>
+      <x:c r="D23" s="2" t="str">
+        <x:v>Shi, Mingrui, Haozhen Situ,</x:v>
+      </x:c>
+      <x:c r="E23" s="2" t="str">
+        <x:v>https://iopscience.iop.org/article/10.1088/1402-4896/ad3e3d/meta</x:v>
+      </x:c>
+      <x:c r="F23" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="24">
+      <x:c r="A24" s="2" t="str">
+        <x:v>Optimization enabled Deep Quantum Neural Network for weed classification and density estimation</x:v>
+      </x:c>
+      <x:c r="B24" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C24" s="2" t="str">
+        <x:v>Expert Systems with Applications </x:v>
+      </x:c>
+      <x:c r="D24" s="2" t="str">
+        <x:v>Veeragandham, Syamasudha,</x:v>
+      </x:c>
+      <x:c r="E24" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0957417423031810</x:v>
+      </x:c>
+      <x:c r="F24" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="25">
+      <x:c r="A25" s="2" t="str">
+        <x:v>Estimating quantum mutual information through a quantum neural network</x:v>
+      </x:c>
+      <x:c r="B25" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C25" s="2" t="str">
+        <x:v>Quantum Information Processing</x:v>
+      </x:c>
+      <x:c r="D25" s="2" t="str">
+        <x:v>Shin, Myeongjin</x:v>
+      </x:c>
+      <x:c r="E25" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11128-023-04253-1</x:v>
+      </x:c>
+      <x:c r="F25" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="26">
+      <x:c r="A26" s="2" t="str">
+        <x:v>Superposition-enhanced quantum neural network for multi-class image classification</x:v>
+      </x:c>
+      <x:c r="B26" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C26" s="2" t="str">
+        <x:v>Journal of Physics </x:v>
+      </x:c>
+      <x:c r="D26" s="2" t="str">
+        <x:v>Bai, Qi, and Xianliang</x:v>
+      </x:c>
+      <x:c r="E26" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0577907324001151</x:v>
+      </x:c>
+      <x:c r="F26" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="27">
+      <x:c r="A27" s="2" t="str">
+        <x:v>Restricting to the chip architecture maintains the quantum neural network accuracy</x:v>
+      </x:c>
+      <x:c r="B27" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C27" s="2" t="str">
+        <x:v>Quantum Information Processing</x:v>
+      </x:c>
+      <x:c r="D27" s="2" t="str">
+        <x:v>Friedrich, Lucas,</x:v>
+      </x:c>
+      <x:c r="E27" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11128-024-04336-7</x:v>
+      </x:c>
+      <x:c r="F27" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="28">
+      <x:c r="A28" s="2" t="str">
         <x:v>Quantum neural network with ensemble learning to mitigate barren plateaus and cost function concentration
 </x:v>
       </x:c>
-      <x:c r="B22" s="2" t="n">
+      <x:c r="B28" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C22" s="2" t="str">
+      <x:c r="C28" s="2" t="str">
         <x:v>arXiv preprint</x:v>
       </x:c>
-      <x:c r="D22" s="2" t="str">
+      <x:c r="D28" s="2" t="str">
         <x:v>Friedrich, Lucas,Friedrich</x:v>
       </x:c>
-      <x:c r="E22" s="2" t="str">
+      <x:c r="E28" s="2" t="str">
         <x:v>https://arxiv.org/abs/2402.06026</x:v>
       </x:c>
-      <x:c r="F22" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="23">
-      <x:c r="A23" s="2" t="str">
+      <x:c r="F28" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="29">
+      <x:c r="A29" s="2" t="str">
         <x:v>Theory for equivariant quantum neural networks</x:v>
       </x:c>
-      <x:c r="B23" s="2" t="n">
+      <x:c r="B29" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C23" s="2" t="str">
+      <x:c r="C29" s="2" t="str">
         <x:v>PRX Quantum </x:v>
       </x:c>
-      <x:c r="D23" s="2" t="str">
+      <x:c r="D29" s="2" t="str">
         <x:v>Nguyen, Quynh</x:v>
       </x:c>
-      <x:c r="E23" s="2" t="str">
+      <x:c r="E29" s="2" t="str">
         <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.5.020328</x:v>
       </x:c>
-      <x:c r="F23" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="24">
-      <x:c r="A24" s="2" t="str">
+      <x:c r="F29" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="30">
+      <x:c r="A30" s="2" t="str">
         <x:v>Quantum Neural Network Training of a Repeater Node</x:v>
       </x:c>
-      <x:c r="B24" s="2" t="n">
+      <x:c r="B30" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C24" s="2" t="str">
+      <x:c r="C30" s="2" t="str">
         <x:v>arXiv preprint </x:v>
       </x:c>
-      <x:c r="D24" s="2" t="str">
+      <x:c r="D30" s="2" t="str">
         <x:v>Fuentealba, Diego</x:v>
       </x:c>
-      <x:c r="E24" s="2" t="str">
+      <x:c r="E30" s="2" t="str">
         <x:v>https://arxiv.org/abs/2408.04709</x:v>
       </x:c>
-      <x:c r="F24" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="25">
-      <x:c r="A25" s="2" t="str">
+      <x:c r="F30" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="31">
+      <x:c r="A31" s="2" t="str">
         <x:v>A quantum neural network framework for scalable quantum circuit approximation of unitary matrices
 </x:v>
       </x:c>
-      <x:c r="B25" s="2" t="n">
+      <x:c r="B31" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C25" s="2" t="str">
+      <x:c r="C31" s="2" t="str">
         <x:v>arXiv preprint </x:v>
       </x:c>
-      <x:c r="D25" s="2" t="str">
+      <x:c r="D31" s="2" t="str">
         <x:v>Sarkar, Rohit Sarma, </x:v>
       </x:c>
-      <x:c r="E25" s="2" t="str">
+      <x:c r="E31" s="2" t="str">
         <x:v>https://arxiv.org/abs/2405.00012</x:v>
       </x:c>
-      <x:c r="F25" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="26">
-      <x:c r="A26" s="2" t="str">
+      <x:c r="F31" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="32">
+      <x:c r="A32" s="2" t="str">
         <x:v>Quantum neural estimation of entropies
 </x:v>
       </x:c>
-      <x:c r="B26" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C26" s="2" t="str">
-        <x:v>Physical Review </x:v>
-      </x:c>
-      <x:c r="D26" s="2" t="str">
-        <x:v>Goldfeld, Ziv, </x:v>
-      </x:c>
-      <x:c r="E26" s="2" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.109.032431</x:v>
-      </x:c>
-      <x:c r="F26" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="27">
-      <x:c r="A27" s="2" t="str">
-        <x:v>Enforcing exact permutation and rotational symmetries in the application of quantum neural network on point cloud datasets</x:v>
-      </x:c>
-      <x:c r="B27" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C27" s="2" t="str">
-        <x:v>arXiv preprint </x:v>
-      </x:c>
-      <x:c r="D27" s="2" t="str">
-        <x:v>Li, Zhelun, Lento Nagano,</x:v>
-      </x:c>
-      <x:c r="E27" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2405.11150</x:v>
-      </x:c>
-      <x:c r="F27" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="28">
-      <x:c r="A28" s="2" t="str">
-        <x:v>Quantum Neural Network Software Testing, Analysis, and Code Optimization for Advanced IoT Systems: Design, Implementation, and Visualization</x:v>
-      </x:c>
-      <x:c r="B28" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C28" s="2" t="str">
-        <x:v>arXiv preprint </x:v>
-      </x:c>
-      <x:c r="D28" s="2" t="str">
-        <x:v>Park, Soohyun,</x:v>
-      </x:c>
-      <x:c r="E28" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2401.10914</x:v>
-      </x:c>
-      <x:c r="F28" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="29">
-      <x:c r="A29" s="2" t="str">
-        <x:v>Quantum neural networks for power flow analysis</x:v>
-      </x:c>
-      <x:c r="B29" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C29" s="2" t="str">
-        <x:v>Electric Power Systems Research</x:v>
-      </x:c>
-      <x:c r="D29" s="2" t="str">
-        <x:v>Kaseb, Zeynab</x:v>
-      </x:c>
-      <x:c r="E29" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S0378779624005637</x:v>
-      </x:c>
-      <x:c r="F29" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="30">
-      <x:c r="A30" s="2" t="str">
-        <x:v>Hybrid parameters for fluid identification using an enhanced quantum neural network in a tight reservoir</x:v>
-      </x:c>
-      <x:c r="B30" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C30" s="2" t="str">
-        <x:v>Scientific Reports </x:v>
-      </x:c>
-      <x:c r="D30" s="2" t="str">
-        <x:v>Luo, Dejiang</x:v>
-      </x:c>
-      <x:c r="E30" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41598-023-50455-z</x:v>
-      </x:c>
-      <x:c r="F30" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="31">
-      <x:c r="A31" s="2" t="str">
-        <x:v>Quantum optimization for training quantum neural networks</x:v>
-      </x:c>
-      <x:c r="B31" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C31" s="2" t="str">
-        <x:v>Quantum Machine Intelligence</x:v>
-      </x:c>
-      <x:c r="D31" s="2" t="str">
-        <x:v>Liao, Yidong, Min-Hsiu Hsieh</x:v>
-      </x:c>
-      <x:c r="E31" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-024-00169-w</x:v>
-      </x:c>
-      <x:c r="F31" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="32">
-      <x:c r="A32" s="2" t="str">
-        <x:v>Statistical analysis of quantum state learning process in quantum neural networks</x:v>
-      </x:c>
       <x:c r="B32" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C32" s="2" t="str">
-        <x:v>Advances in Neural Information Processing Systems</x:v>
+        <x:v>Physical Review </x:v>
       </x:c>
       <x:c r="D32" s="2" t="str">
-        <x:v>Zhang, Hao-kai, </x:v>
+        <x:v>Goldfeld, Ziv, </x:v>
       </x:c>
       <x:c r="E32" s="2" t="str">
-        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/68efc144ad3b41108f779b51b9fb1300-Abstract-Conference.html</x:v>
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.109.032431</x:v>
       </x:c>
       <x:c r="F32" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2432,19 +2432,19 @@
     </x:row>
     <x:row r="33">
       <x:c r="A33" s="2" t="str">
-        <x:v>Hyperparameter importance and optimization of quantum neural networks across small datasets</x:v>
+        <x:v>Enforcing exact permutation and rotational symmetries in the application of quantum neural network on point cloud datasets</x:v>
       </x:c>
       <x:c r="B33" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C33" s="2" t="str">
-        <x:v>Machine Learning </x:v>
+        <x:v>arXiv preprint </x:v>
       </x:c>
       <x:c r="D33" s="2" t="str">
-        <x:v>Moussa, Charles, </x:v>
+        <x:v>Li, Zhelun, Lento Nagano,</x:v>
       </x:c>
       <x:c r="E33" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s10994-023-06389-8</x:v>
+        <x:v>https://arxiv.org/abs/2405.11150</x:v>
       </x:c>
       <x:c r="F33" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2452,140 +2452,140 @@
     </x:row>
     <x:row r="34">
       <x:c r="A34" s="2" t="str">
+        <x:v>Quantum Neural Network Software Testing, Analysis, and Code Optimization for Advanced IoT Systems: Design, Implementation, and Visualization</x:v>
+      </x:c>
+      <x:c r="B34" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C34" s="2" t="str">
+        <x:v>arXiv preprint </x:v>
+      </x:c>
+      <x:c r="D34" s="2" t="str">
+        <x:v>Park, Soohyun,</x:v>
+      </x:c>
+      <x:c r="E34" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2401.10914</x:v>
+      </x:c>
+      <x:c r="F34" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="35">
+      <x:c r="A35" s="2" t="str">
+        <x:v>Quantum neural networks for power flow analysis</x:v>
+      </x:c>
+      <x:c r="B35" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C35" s="2" t="str">
+        <x:v>Electric Power Systems Research</x:v>
+      </x:c>
+      <x:c r="D35" s="2" t="str">
+        <x:v>Kaseb, Zeynab</x:v>
+      </x:c>
+      <x:c r="E35" s="2" t="str">
+        <x:v>https://www.sciencedirect.com/science/article/pii/S0378779624005637</x:v>
+      </x:c>
+      <x:c r="F35" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="36">
+      <x:c r="A36" s="2" t="str">
+        <x:v>Hybrid parameters for fluid identification using an enhanced quantum neural network in a tight reservoir</x:v>
+      </x:c>
+      <x:c r="B36" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C36" s="2" t="str">
+        <x:v>Scientific Reports </x:v>
+      </x:c>
+      <x:c r="D36" s="2" t="str">
+        <x:v>Luo, Dejiang</x:v>
+      </x:c>
+      <x:c r="E36" s="2" t="str">
+        <x:v>https://www.nature.com/articles/s41598-023-50455-z</x:v>
+      </x:c>
+      <x:c r="F36" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="37">
+      <x:c r="A37" s="2" t="str">
+        <x:v>Quantum optimization for training quantum neural networks</x:v>
+      </x:c>
+      <x:c r="B37" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C37" s="2" t="str">
+        <x:v>Quantum Machine Intelligence</x:v>
+      </x:c>
+      <x:c r="D37" s="2" t="str">
+        <x:v>Liao, Yidong, Min-Hsiu Hsieh</x:v>
+      </x:c>
+      <x:c r="E37" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s42484-024-00169-w</x:v>
+      </x:c>
+      <x:c r="F37" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="38">
+      <x:c r="A38" s="2" t="str">
+        <x:v>Statistical analysis of quantum state learning process in quantum neural networks</x:v>
+      </x:c>
+      <x:c r="B38" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C38" s="2" t="str">
+        <x:v>Advances in Neural Information Processing Systems</x:v>
+      </x:c>
+      <x:c r="D38" s="2" t="str">
+        <x:v>Zhang, Hao-kai, </x:v>
+      </x:c>
+      <x:c r="E38" s="2" t="str">
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2023/hash/68efc144ad3b41108f779b51b9fb1300-Abstract-Conference.html</x:v>
+      </x:c>
+      <x:c r="F38" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="39">
+      <x:c r="A39" s="2" t="str">
+        <x:v>Hyperparameter importance and optimization of quantum neural networks across small datasets</x:v>
+      </x:c>
+      <x:c r="B39" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C39" s="2" t="str">
+        <x:v>Machine Learning </x:v>
+      </x:c>
+      <x:c r="D39" s="2" t="str">
+        <x:v>Moussa, Charles, </x:v>
+      </x:c>
+      <x:c r="E39" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s10994-023-06389-8</x:v>
+      </x:c>
+      <x:c r="F39" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="40">
+      <x:c r="A40" s="2" t="str">
         <x:v>VIOLET: Visual Analytics for Explainable Quantum Neural Networks
 </x:v>
       </x:c>
-      <x:c r="B34" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C34" s="2" t="str">
-        <x:v>IEEE Transactions on Visualization and Computer Graphics </x:v>
-      </x:c>
-      <x:c r="D34" s="2" t="str">
-        <x:v>Ruan, Shaolun</x:v>
-      </x:c>
-      <x:c r="E34" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10507082</x:v>
-      </x:c>
-      <x:c r="F34" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="35">
-      <x:c r="A35" s="2" t="str">
-        <x:v>Explainable hybrid quantum neural networks for analyzing the influence of tweets on stock price prediction</x:v>
-      </x:c>
-      <x:c r="B35" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C35" s="2" t="str">
-        <x:v>Computers and Electrical Engineering </x:v>
-      </x:c>
-      <x:c r="D35" s="2" t="str">
-        <x:v>Gandhudi, Manoranjan</x:v>
-      </x:c>
-      <x:c r="E35" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0045790624002301</x:v>
-      </x:c>
-      <x:c r="F35" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="36">
-      <x:c r="A36" s="2" t="str">
-        <x:v>Network Anomaly Detection Using Quantum Neural Networks on Noisy Quantum Computers.</x:v>
-      </x:c>
-      <x:c r="B36" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C36" s="2" t="str">
-        <x:v>IEEE Transactions on Quantum Engineering </x:v>
-      </x:c>
-      <x:c r="D36" s="2" t="str">
-        <x:v>Kukliansky, Alon</x:v>
-      </x:c>
-      <x:c r="E36" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10415536</x:v>
-      </x:c>
-      <x:c r="F36" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="37">
-      <x:c r="A37" s="2" t="str">
-        <x:v>Deep Q-learning with hybrid quantum neural network on solving maze problems</x:v>
-      </x:c>
-      <x:c r="B37" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C37" s="2" t="str">
-        <x:v>Quantum Machine Intelligence</x:v>
-      </x:c>
-      <x:c r="D37" s="2" t="str">
-        <x:v>Chen, Hao-Yuan, </x:v>
-      </x:c>
-      <x:c r="E37" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-023-00137-w</x:v>
-      </x:c>
-      <x:c r="F37" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="38">
-      <x:c r="A38" s="2" t="str">
-        <x:v>Theoretical guarantees for permutation-equivariant quantum neural networks</x:v>
-      </x:c>
-      <x:c r="B38" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C38" s="2" t="str">
-        <x:v>npj Quantum Information </x:v>
-      </x:c>
-      <x:c r="D38" s="2" t="str">
-        <x:v>Schatzki, Louis, </x:v>
-      </x:c>
-      <x:c r="E38" s="2" t="str">
-        <x:v>https://www.nature.com/articles/s41534-024-00804-1</x:v>
-      </x:c>
-      <x:c r="F38" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="39">
-      <x:c r="A39" s="2" t="str">
-        <x:v>Quantum mesh neural network model in precise image diagnosing</x:v>
-      </x:c>
-      <x:c r="B39" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C39" s="2" t="str">
-        <x:v>Optical and Quantum Electronics</x:v>
-      </x:c>
-      <x:c r="D39" s="2" t="str">
-        <x:v>Suneel, Sajja, </x:v>
-      </x:c>
-      <x:c r="E39" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11082-023-06245-y</x:v>
-      </x:c>
-      <x:c r="F39" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="40">
-      <x:c r="A40" s="2" t="str">
-        <x:v>Neural-network quantum states for many-body physics</x:v>
-      </x:c>
       <x:c r="B40" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C40" s="2" t="str">
-        <x:v>arXiv preprint </x:v>
+        <x:v>IEEE Transactions on Visualization and Computer Graphics </x:v>
       </x:c>
       <x:c r="D40" s="2" t="str">
-        <x:v>Medvidović, Matija</x:v>
+        <x:v>Ruan, Shaolun</x:v>
       </x:c>
       <x:c r="E40" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2402.11014</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10507082</x:v>
       </x:c>
       <x:c r="F40" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2593,19 +2593,19 @@
     </x:row>
     <x:row r="41">
       <x:c r="A41" s="2" t="str">
-        <x:v>A Novel Quantum Neural Network Approach to Combating Fake Reviews</x:v>
+        <x:v>Explainable hybrid quantum neural networks for analyzing the influence of tweets on stock price prediction</x:v>
       </x:c>
       <x:c r="B41" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C41" s="2" t="str">
-        <x:v>International Journal of Networked and Distributed Computing</x:v>
+        <x:v>Computers and Electrical Engineering </x:v>
       </x:c>
       <x:c r="D41" s="2" t="str">
-        <x:v>Bikku, Thulasi, </x:v>
+        <x:v>Gandhudi, Manoranjan</x:v>
       </x:c>
       <x:c r="E41" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s44227-024-00028-x</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0045790624002301</x:v>
       </x:c>
       <x:c r="F41" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2613,19 +2613,19 @@
     </x:row>
     <x:row r="42">
       <x:c r="A42" s="2" t="str">
-        <x:v>Generative invertible quantum neural networks</x:v>
+        <x:v>Network Anomaly Detection Using Quantum Neural Networks on Noisy Quantum Computers.</x:v>
       </x:c>
       <x:c r="B42" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C42" s="2" t="str">
-        <x:v>SciPost Physics </x:v>
+        <x:v>IEEE Transactions on Quantum Engineering </x:v>
       </x:c>
       <x:c r="D42" s="2" t="str">
-        <x:v>Rousselot, Armand,</x:v>
+        <x:v>Kukliansky, Alon</x:v>
       </x:c>
       <x:c r="E42" s="2" t="str">
-        <x:v>https://www.scipost.org/SciPostPhys.16.6.146?acad_field_slug=astronomy</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10415536</x:v>
       </x:c>
       <x:c r="F42" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2633,201 +2633,201 @@
     </x:row>
     <x:row r="43">
       <x:c r="A43" s="2" t="str">
+        <x:v>Deep Q-learning with hybrid quantum neural network on solving maze problems</x:v>
+      </x:c>
+      <x:c r="B43" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C43" s="2" t="str">
+        <x:v>Quantum Machine Intelligence</x:v>
+      </x:c>
+      <x:c r="D43" s="2" t="str">
+        <x:v>Chen, Hao-Yuan, </x:v>
+      </x:c>
+      <x:c r="E43" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s42484-023-00137-w</x:v>
+      </x:c>
+      <x:c r="F43" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44">
+      <x:c r="A44" s="2" t="str">
+        <x:v>Theoretical guarantees for permutation-equivariant quantum neural networks</x:v>
+      </x:c>
+      <x:c r="B44" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C44" s="2" t="str">
+        <x:v>npj Quantum Information </x:v>
+      </x:c>
+      <x:c r="D44" s="2" t="str">
+        <x:v>Schatzki, Louis, </x:v>
+      </x:c>
+      <x:c r="E44" s="2" t="str">
+        <x:v>https://www.nature.com/articles/s41534-024-00804-1</x:v>
+      </x:c>
+      <x:c r="F44" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45">
+      <x:c r="A45" s="2" t="str">
+        <x:v>Quantum mesh neural network model in precise image diagnosing</x:v>
+      </x:c>
+      <x:c r="B45" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C45" s="2" t="str">
+        <x:v>Optical and Quantum Electronics</x:v>
+      </x:c>
+      <x:c r="D45" s="2" t="str">
+        <x:v>Suneel, Sajja, </x:v>
+      </x:c>
+      <x:c r="E45" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11082-023-06245-y</x:v>
+      </x:c>
+      <x:c r="F45" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46">
+      <x:c r="A46" s="2" t="str">
+        <x:v>Neural-network quantum states for many-body physics</x:v>
+      </x:c>
+      <x:c r="B46" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C46" s="2" t="str">
+        <x:v>arXiv preprint </x:v>
+      </x:c>
+      <x:c r="D46" s="2" t="str">
+        <x:v>Medvidović, Matija</x:v>
+      </x:c>
+      <x:c r="E46" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2402.11014</x:v>
+      </x:c>
+      <x:c r="F46" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47">
+      <x:c r="A47" s="2" t="str">
+        <x:v>A Novel Quantum Neural Network Approach to Combating Fake Reviews</x:v>
+      </x:c>
+      <x:c r="B47" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C47" s="2" t="str">
+        <x:v>International Journal of Networked and Distributed Computing</x:v>
+      </x:c>
+      <x:c r="D47" s="2" t="str">
+        <x:v>Bikku, Thulasi, </x:v>
+      </x:c>
+      <x:c r="E47" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s44227-024-00028-x</x:v>
+      </x:c>
+      <x:c r="F47" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48">
+      <x:c r="A48" s="2" t="str">
+        <x:v>Generative invertible quantum neural networks</x:v>
+      </x:c>
+      <x:c r="B48" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C48" s="2" t="str">
+        <x:v>SciPost Physics </x:v>
+      </x:c>
+      <x:c r="D48" s="2" t="str">
+        <x:v>Rousselot, Armand,</x:v>
+      </x:c>
+      <x:c r="E48" s="2" t="str">
+        <x:v>https://www.scipost.org/SciPostPhys.16.6.146?acad_field_slug=astronomy</x:v>
+      </x:c>
+      <x:c r="F48" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49">
+      <x:c r="A49" s="2" t="str">
         <x:v>Neural-network-encoded variational quantum algorithms
 </x:v>
       </x:c>
-      <x:c r="B43" s="2" t="n">
+      <x:c r="B49" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C43" s="2" t="str">
+      <x:c r="C49" s="2" t="str">
         <x:v>Physical Review Applied </x:v>
       </x:c>
-      <x:c r="D43" s="2" t="str">
+      <x:c r="D49" s="2" t="str">
         <x:v>Miao, Jiaqi, Chang-Yu Hsieh,</x:v>
       </x:c>
-      <x:c r="E43" s="2" t="str">
+      <x:c r="E49" s="2" t="str">
         <x:v>https://journals.aps.org/prapplied/abstract/10.1103/PhysRevApplied.21.014053</x:v>
       </x:c>
-      <x:c r="F43" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="44">
-      <x:c r="A44" s="2" t="str">
+      <x:c r="F49" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50">
+      <x:c r="A50" s="2" t="str">
         <x:v>Enhancing the expressivity of quantum neural networks with residual connections</x:v>
       </x:c>
-      <x:c r="B44" s="2" t="n">
+      <x:c r="B50" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C44" s="2" t="str">
+      <x:c r="C50" s="2" t="str">
         <x:v>Communications Physics</x:v>
       </x:c>
-      <x:c r="D44" s="2" t="str">
+      <x:c r="D50" s="2" t="str">
         <x:v>Wen, Jingwei, </x:v>
       </x:c>
-      <x:c r="E44" s="2" t="str">
+      <x:c r="E50" s="2" t="str">
         <x:v>https://www.nature.com/articles/s42005-024-01719-1</x:v>
       </x:c>
-      <x:c r="F44" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="45">
-      <x:c r="A45" s="2" t="str">
+      <x:c r="F50" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51">
+      <x:c r="A51" s="2" t="str">
         <x:v>ℤ2 × ℤ2 Equivariant Quantum Neural Networks: Benchmarking against Classical Neural Networks</x:v>
       </x:c>
-      <x:c r="B45" s="2" t="n">
+      <x:c r="B51" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C45" s="2" t="str">
+      <x:c r="C51" s="2" t="str">
         <x:v>Axioms</x:v>
       </x:c>
-      <x:c r="D45" s="2" t="str">
+      <x:c r="D51" s="2" t="str">
         <x:v>Dong, Zhongtian,</x:v>
       </x:c>
-      <x:c r="E45" s="2" t="str">
+      <x:c r="E51" s="2" t="str">
         <x:v>https://www.mdpi.com/2075-1680/13/3/188</x:v>
       </x:c>
-      <x:c r="F45" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="46">
-      <x:c r="A46" s="2" t="str">
+      <x:c r="F51" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52">
+      <x:c r="A52" s="2" t="str">
         <x:v>A Quantum Neural Network-Based Approach to Power Quality Disturbances Detection and Recognition
 </x:v>
       </x:c>
-      <x:c r="B46" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C46" s="2" t="str">
-        <x:v>arXiv preprint </x:v>
-      </x:c>
-      <x:c r="D46" s="2" t="str">
-        <x:v>Li, Guo-Dong,</x:v>
-      </x:c>
-      <x:c r="E46" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2406.03081</x:v>
-      </x:c>
-      <x:c r="F46" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="47">
-      <x:c r="A47" s="2" t="str">
-        <x:v>Second-order optimization strategies for neural network quantum states</x:v>
-      </x:c>
-      <x:c r="B47" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C47" s="2" t="str">
-        <x:v>hilosophical Transactions A</x:v>
-      </x:c>
-      <x:c r="D47" s="2" t="str">
-        <x:v>Drissi, M.,</x:v>
-      </x:c>
-      <x:c r="E47" s="2" t="str">
-        <x:v>https://royalsocietypublishing.org/doi/epdf/10.1098/rsta.2024.0057</x:v>
-      </x:c>
-      <x:c r="F47" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="48">
-      <x:c r="A48" s="2" t="str">
-        <x:v>ResQNets: a residual approach for mitigating barren plateaus in quantum neural networks</x:v>
-      </x:c>
-      <x:c r="B48" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C48" s="2" t="str">
-        <x:v>EPJ Quantum Technology</x:v>
-      </x:c>
-      <x:c r="D48" s="2" t="str">
-        <x:v>Kashif, Muhammad,</x:v>
-      </x:c>
-      <x:c r="E48" s="2" t="str">
-        <x:v>https://epjqt.epj.org/articles/epjqt/abs/2024/01/40507_2023_Article_216/40507_2023_Article_216.html</x:v>
-      </x:c>
-      <x:c r="F48" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="49">
-      <x:c r="A49" s="2" t="str">
-        <x:v>Training embedding quantum kernels with data re-uploading quantum neural networks</x:v>
-      </x:c>
-      <x:c r="B49" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C49" s="2" t="str">
-        <x:v>arXiv preprint </x:v>
-      </x:c>
-      <x:c r="D49" s="2" t="str">
-        <x:v>Rodriguez-Grasa, Pablo,</x:v>
-      </x:c>
-      <x:c r="E49" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2401.04642</x:v>
-      </x:c>
-      <x:c r="F49" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="50">
-      <x:c r="A50" s="2" t="str">
-        <x:v>Training Classical Neural Networks by Quantum Machine Learning</x:v>
-      </x:c>
-      <x:c r="B50" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C50" s="2" t="str">
-        <x:v>arXiv preprint </x:v>
-      </x:c>
-      <x:c r="D50" s="2" t="str">
-        <x:v>Liu, Chen-Yu, </x:v>
-      </x:c>
-      <x:c r="E50" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2402.16465</x:v>
-      </x:c>
-      <x:c r="F50" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="51">
-      <x:c r="A51" s="2" t="str">
-        <x:v>Quantum Recurrent Neural Networks: Predicting the Dynamics of Oscillatory and Chaotic Systems</x:v>
-      </x:c>
-      <x:c r="B51" s="2" t="n">
-        <x:v>2024</x:v>
-      </x:c>
-      <x:c r="C51" s="2" t="str">
-        <x:v>Algorithms</x:v>
-      </x:c>
-      <x:c r="D51" s="2" t="str">
-        <x:v>Chen, Yuan, and Abdul Khaliq. "</x:v>
-      </x:c>
-      <x:c r="E51" s="2" t="str">
-        <x:v>https://www.mdpi.com/1999-4893/17/4/163</x:v>
-      </x:c>
-      <x:c r="F51" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="52">
-      <x:c r="A52" s="2" t="str">
-        <x:v>Application of Quantum Recurrent Neural Network in Low Resource Language Text Classification</x:v>
-      </x:c>
       <x:c r="B52" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C52" s="2" t="str">
-        <x:v>IEEE Transactions on Quantum Engineering </x:v>
+        <x:v>arXiv preprint </x:v>
       </x:c>
       <x:c r="D52" s="2" t="str">
-        <x:v>Yu, Wenbin, et al. "</x:v>
+        <x:v>Li, Guo-Dong,</x:v>
       </x:c>
       <x:c r="E52" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10461108</x:v>
+        <x:v>https://arxiv.org/abs/2406.03081</x:v>
       </x:c>
       <x:c r="F52" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2835,19 +2835,19 @@
     </x:row>
     <x:row r="53">
       <x:c r="A53" s="2" t="str">
-        <x:v>An RNN–policy gradient approach for quantum architecture search</x:v>
+        <x:v>Second-order optimization strategies for neural network quantum states</x:v>
       </x:c>
       <x:c r="B53" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
       <x:c r="C53" s="2" t="str">
-        <x:v>Quantum Information Processing </x:v>
+        <x:v>hilosophical Transactions A</x:v>
       </x:c>
       <x:c r="D53" s="2" t="str">
-        <x:v>Wang, Gang, Bang-Hai Wang</x:v>
+        <x:v>Drissi, M.,</x:v>
       </x:c>
       <x:c r="E53" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11128-024-04393-y</x:v>
+        <x:v>https://royalsocietypublishing.org/doi/epdf/10.1098/rsta.2024.0057</x:v>
       </x:c>
       <x:c r="F53" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2855,140 +2855,140 @@
     </x:row>
     <x:row r="54">
       <x:c r="A54" s="2" t="str">
+        <x:v>ResQNets: a residual approach for mitigating barren plateaus in quantum neural networks</x:v>
+      </x:c>
+      <x:c r="B54" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C54" s="2" t="str">
+        <x:v>EPJ Quantum Technology</x:v>
+      </x:c>
+      <x:c r="D54" s="2" t="str">
+        <x:v>Kashif, Muhammad,</x:v>
+      </x:c>
+      <x:c r="E54" s="2" t="str">
+        <x:v>https://epjqt.epj.org/articles/epjqt/abs/2024/01/40507_2023_Article_216/40507_2023_Article_216.html</x:v>
+      </x:c>
+      <x:c r="F54" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55">
+      <x:c r="A55" s="2" t="str">
+        <x:v>Training embedding quantum kernels with data re-uploading quantum neural networks</x:v>
+      </x:c>
+      <x:c r="B55" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C55" s="2" t="str">
+        <x:v>arXiv preprint </x:v>
+      </x:c>
+      <x:c r="D55" s="2" t="str">
+        <x:v>Rodriguez-Grasa, Pablo,</x:v>
+      </x:c>
+      <x:c r="E55" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2401.04642</x:v>
+      </x:c>
+      <x:c r="F55" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56">
+      <x:c r="A56" s="2" t="str">
+        <x:v>Training Classical Neural Networks by Quantum Machine Learning</x:v>
+      </x:c>
+      <x:c r="B56" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C56" s="2" t="str">
+        <x:v>arXiv preprint </x:v>
+      </x:c>
+      <x:c r="D56" s="2" t="str">
+        <x:v>Liu, Chen-Yu, </x:v>
+      </x:c>
+      <x:c r="E56" s="2" t="str">
+        <x:v>https://arxiv.org/abs/2402.16465</x:v>
+      </x:c>
+      <x:c r="F56" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57">
+      <x:c r="A57" s="2" t="str">
+        <x:v>Quantum Recurrent Neural Networks: Predicting the Dynamics of Oscillatory and Chaotic Systems</x:v>
+      </x:c>
+      <x:c r="B57" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C57" s="2" t="str">
+        <x:v>Algorithms</x:v>
+      </x:c>
+      <x:c r="D57" s="2" t="str">
+        <x:v>Chen, Yuan, and Abdul Khaliq. "</x:v>
+      </x:c>
+      <x:c r="E57" s="2" t="str">
+        <x:v>https://www.mdpi.com/1999-4893/17/4/163</x:v>
+      </x:c>
+      <x:c r="F57" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58">
+      <x:c r="A58" s="2" t="str">
+        <x:v>Application of Quantum Recurrent Neural Network in Low Resource Language Text Classification</x:v>
+      </x:c>
+      <x:c r="B58" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C58" s="2" t="str">
+        <x:v>IEEE Transactions on Quantum Engineering </x:v>
+      </x:c>
+      <x:c r="D58" s="2" t="str">
+        <x:v>Yu, Wenbin, et al. "</x:v>
+      </x:c>
+      <x:c r="E58" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10461108</x:v>
+      </x:c>
+      <x:c r="F58" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59">
+      <x:c r="A59" s="2" t="str">
+        <x:v>An RNN–policy gradient approach for quantum architecture search</x:v>
+      </x:c>
+      <x:c r="B59" s="2" t="n">
+        <x:v>2024</x:v>
+      </x:c>
+      <x:c r="C59" s="2" t="str">
+        <x:v>Quantum Information Processing </x:v>
+      </x:c>
+      <x:c r="D59" s="2" t="str">
+        <x:v>Wang, Gang, Bang-Hai Wang</x:v>
+      </x:c>
+      <x:c r="E59" s="2" t="str">
+        <x:v>https://link.springer.com/article/10.1007/s11128-024-04393-y</x:v>
+      </x:c>
+      <x:c r="F59" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="60">
+      <x:c r="A60" s="2" t="str">
         <x:v>Applying Hybrid Quantum LSTM for Indoor Localization Based on RSSI
 </x:v>
       </x:c>
-      <x:c r="B54" s="2" t="n">
+      <x:c r="B60" s="2" t="n">
         <x:v>2024</x:v>
       </x:c>
-      <x:c r="C54" s="2" t="str">
+      <x:c r="C60" s="2" t="str">
         <x:v>EEE International Conference on Acoustics, Speech and Signal Processing (ICASSP)</x:v>
       </x:c>
-      <x:c r="D54" s="2" t="str">
+      <x:c r="D60" s="2" t="str">
         <x:v>Chien, S. F., et al. </x:v>
       </x:c>
-      <x:c r="E54" s="2" t="str">
+      <x:c r="E60" s="2" t="str">
         <x:v>https://ieeexplore.ieee.org/abstract/document/10447032</x:v>
-      </x:c>
-      <x:c r="F54" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="55">
-      <x:c r="A55" s="2" t="str">
-        <x:v>Quantum Neural Network for Quantum Neural Computing</x:v>
-      </x:c>
-      <x:c r="B55" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C55" s="2" t="str">
-        <x:v>Research A SCIENCE PARTNER JOURNAL</x:v>
-      </x:c>
-      <x:c r="D55" s="2" t="str">
-        <x:v>Min-Gang Zhou, Zhi-Ping Liu, Hua-Lei Yin, Chen-Long Li, Tong-Kai Xu, and Zeng-Bing Chen </x:v>
-      </x:c>
-      <x:c r="E55" s="2" t="str">
-        <x:v>https://doi.org/10.34133/research.0134</x:v>
-      </x:c>
-      <x:c r="F55" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="56">
-      <x:c r="A56" s="2" t="str">
-        <x:v>QNMF: A quantum neural network based multimodal fusion system for intelligent diagnosis</x:v>
-      </x:c>
-      <x:c r="B56" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C56" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
-      </x:c>
-      <x:c r="D56" s="2" t="str">
-        <x:v>Zhiguo Qu, Yang Li b, Prayag Tiwari</x:v>
-      </x:c>
-      <x:c r="E56" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.inffus.2023.101913</x:v>
-      </x:c>
-      <x:c r="F56" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="57">
-      <x:c r="A57" s="2" t="str">
-        <x:v>Hybrid Quantum Neural Network for Drug Response Prediction</x:v>
-      </x:c>
-      <x:c r="B57" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C57" s="2" t="str">
-        <x:v>MDPI</x:v>
-      </x:c>
-      <x:c r="D57" s="2" t="str">
-        <x:v>Asel Sagingalieva, Mohammad Kordzanganeh, Nurbolat Kenbayev,Daria Kosichkina, Tatiana Tomashuk, Alexey Melnikov</x:v>
-      </x:c>
-      <x:c r="E57" s="2" t="str">
-        <x:v>https://doi.org/10.3390/cancers15102705</x:v>
-      </x:c>
-      <x:c r="F57" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="58">
-      <x:c r="A58" s="2" t="str">
-        <x:v>Quantum neural network cost function concentration dependency on the parametrization expressivity</x:v>
-      </x:c>
-      <x:c r="B58" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C58" s="2" t="str">
-        <x:v>Scientific report</x:v>
-      </x:c>
-      <x:c r="D58" s="2" t="str">
-        <x:v>Lucas Friedrich, Jonas Maziero</x:v>
-      </x:c>
-      <x:c r="E58" s="2" t="str">
-        <x:v>https://doi.org/10.1038/s41598-023-37003-5</x:v>
-      </x:c>
-      <x:c r="F58" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="59">
-      <x:c r="A59" s="2" t="str">
-        <x:v>Quantum phase detection generalization from marginal quantum neural network models</x:v>
-      </x:c>
-      <x:c r="B59" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C59" s="2" t="str">
-        <x:v>APS</x:v>
-      </x:c>
-      <x:c r="D59" s="2" t="str">
-        <x:v>Saverio Monaco, Oriel Kiss, Antonio Mandarino, Sofia Vallecorsa, Michele Grossi</x:v>
-      </x:c>
-      <x:c r="E59" s="2" t="str">
-        <x:v>https://doi.org/10.1103/PhysRevB.107.L081105</x:v>
-      </x:c>
-      <x:c r="F59" s="2" t="str">
-        <x:v>QNN</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="60">
-      <x:c r="A60" s="2" t="str">
-        <x:v>IoMT-Based Smart Healthcare Detection System Driven by Quantum Blockchain and Quantum Neural Network</x:v>
-      </x:c>
-      <x:c r="B60" s="2" t="n">
-        <x:v>2023</x:v>
-      </x:c>
-      <x:c r="C60" s="2" t="str">
-        <x:v>IEEE Xplore: IEEE Journal of Biomedical and Health Informatics</x:v>
-      </x:c>
-      <x:c r="D60" s="2" t="str">
-        <x:v>Zhiguo Qu, Wenke Shi, Bo Liu, Deepak Gupta, Prayag Tiwari</x:v>
-      </x:c>
-      <x:c r="E60" s="2" t="str">
-        <x:v>10.1109/jbhi.2023.3288199</x:v>
       </x:c>
       <x:c r="F60" s="2" t="str">
         <x:v>QNN</x:v>
@@ -2996,19 +2996,19 @@
     </x:row>
     <x:row r="61">
       <x:c r="A61" s="2" t="str">
-        <x:v>Quantum Neural Network Based Distinguisher on SPECK-32/64</x:v>
+        <x:v>Quantum Neural Network for Quantum Neural Computing</x:v>
       </x:c>
       <x:c r="B61" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C61" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>Research A SCIENCE PARTNER JOURNAL</x:v>
       </x:c>
       <x:c r="D61" s="2" t="str">
-        <x:v> Hyunji Kim, Kyungbae Jang, Sejin Lim, Yeajun Kang, Wonwoong Kim, Hwajeong Seo</x:v>
+        <x:v>Min-Gang Zhou, Zhi-Ping Liu, Hua-Lei Yin, Chen-Long Li, Tong-Kai Xu, and Zeng-Bing Chen </x:v>
       </x:c>
       <x:c r="E61" s="2" t="str">
-        <x:v>https://doi.org/10.3390/s23125683</x:v>
+        <x:v>https://doi.org/10.34133/research.0134</x:v>
       </x:c>
       <x:c r="F61" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3016,7 +3016,7 @@
     </x:row>
     <x:row r="62">
       <x:c r="A62" s="2" t="str">
-        <x:v>Optimization enabled Deep Quantum Neural Network for weed classification and density estimation</x:v>
+        <x:v>QNMF: A quantum neural network based multimodal fusion system for intelligent diagnosis</x:v>
       </x:c>
       <x:c r="B62" s="2" t="n">
         <x:v>2023</x:v>
@@ -3025,10 +3025,10 @@
         <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D62" s="2" t="str">
-        <x:v>Syamasudha Veeragandham, H. Santhi</x:v>
+        <x:v>Zhiguo Qu, Yang Li b, Prayag Tiwari</x:v>
       </x:c>
       <x:c r="E62" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.eswa.2023.122679</x:v>
+        <x:v>https://doi.org/10.1016/j.inffus.2023.101913</x:v>
       </x:c>
       <x:c r="F62" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3036,19 +3036,19 @@
     </x:row>
     <x:row r="63">
       <x:c r="A63" s="2" t="str">
-        <x:v>Approximately Equivariant Quantum Neural Network for p4m Group Symmetries in Images</x:v>
+        <x:v>Hybrid Quantum Neural Network for Drug Response Prediction</x:v>
       </x:c>
       <x:c r="B63" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C63" s="2" t="str">
-        <x:v>IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D63" s="2" t="str">
-        <x:v>Su Yeon Chang, Michele Grossi, Bertrand Le Saux, Sofia Vallecorsa</x:v>
+        <x:v>Asel Sagingalieva, Mohammad Kordzanganeh, Nurbolat Kenbayev,Daria Kosichkina, Tatiana Tomashuk, Alexey Melnikov</x:v>
       </x:c>
       <x:c r="E63" s="2" t="str">
-        <x:v>https://doi.org/10.1109/QCE57702.2023.00033</x:v>
+        <x:v>https://doi.org/10.3390/cancers15102705</x:v>
       </x:c>
       <x:c r="F63" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3056,19 +3056,19 @@
     </x:row>
     <x:row r="64">
       <x:c r="A64" s="2" t="str">
-        <x:v>Estimating quantum mutual information through a quantum neural network</x:v>
+        <x:v>Quantum neural network cost function concentration dependency on the parametrization expressivity</x:v>
       </x:c>
       <x:c r="B64" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C64" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>Scientific report</x:v>
       </x:c>
       <x:c r="D64" s="2" t="str">
-        <x:v>Myeongjin Shin, Junseo Lee &amp; Kabgyun Jeong</x:v>
+        <x:v>Lucas Friedrich, Jonas Maziero</x:v>
       </x:c>
       <x:c r="E64" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s11128-023-04253-1</x:v>
+        <x:v>https://doi.org/10.1038/s41598-023-37003-5</x:v>
       </x:c>
       <x:c r="F64" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3076,19 +3076,19 @@
     </x:row>
     <x:row r="65">
       <x:c r="A65" s="2" t="str">
-        <x:v>Federated Quantum Neural Network With Quantum Teleportation for Resource Optimization in Future Wireless Communication</x:v>
+        <x:v>Quantum phase detection generalization from marginal quantum neural network models</x:v>
       </x:c>
       <x:c r="B65" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C65" s="2" t="str">
-        <x:v>IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
+        <x:v>APS</x:v>
       </x:c>
       <x:c r="D65" s="2" t="str">
-        <x:v>Bhaskara Narottama, Soo Young Shin</x:v>
+        <x:v>Saverio Monaco, Oriel Kiss, Antonio Mandarino, Sofia Vallecorsa, Michele Grossi</x:v>
       </x:c>
       <x:c r="E65" s="2" t="str">
-        <x:v>https://doi.org/10.1109/TVT.2023.3280459</x:v>
+        <x:v>https://doi.org/10.1103/PhysRevB.107.L081105</x:v>
       </x:c>
       <x:c r="F65" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3096,19 +3096,19 @@
     </x:row>
     <x:row r="66">
       <x:c r="A66" s="2" t="str">
-        <x:v>Intrusion detection model using optimized quantum neural network and elliptical curve cryptography for data security</x:v>
+        <x:v>IoMT-Based Smart Healthcare Detection System Driven by Quantum Blockchain and Quantum Neural Network</x:v>
       </x:c>
       <x:c r="B66" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C66" s="2" t="str">
-        <x:v>ScienceDirect</x:v>
+        <x:v>IEEE Xplore: IEEE Journal of Biomedical and Health Informatics</x:v>
       </x:c>
       <x:c r="D66" s="2" t="str">
-        <x:v>Heba Kadry, Ahmed Farouk, Elnomery A. Zanaty, Omar Reyad</x:v>
+        <x:v>Zhiguo Qu, Wenke Shi, Bo Liu, Deepak Gupta, Prayag Tiwari</x:v>
       </x:c>
       <x:c r="E66" s="2" t="str">
-        <x:v>https://doi.org/10.1016/j.aej.2023.03.072</x:v>
+        <x:v>10.1109/jbhi.2023.3288199</x:v>
       </x:c>
       <x:c r="F66" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3116,19 +3116,19 @@
     </x:row>
     <x:row r="67">
       <x:c r="A67" s="2" t="str">
-        <x:v>Quantum Neural Network Inspired Hardware Adaptable Ansatz for Efficient Quantum Simulation of Chemical Systems</x:v>
+        <x:v>Quantum Neural Network Based Distinguisher on SPECK-32/64</x:v>
       </x:c>
       <x:c r="B67" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C67" s="2" t="str">
-        <x:v>Chemical Theory and Computation</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D67" s="2" t="str">
-        <x:v>Xiongzhi Zeng, Yi FanJie Liu, Zhenyu Li, Jinlong Yang</x:v>
+        <x:v> Hyunji Kim, Kyungbae Jang, Sejin Lim, Yeajun Kang, Wonwoong Kim, Hwajeong Seo</x:v>
       </x:c>
       <x:c r="E67" s="2" t="str">
-        <x:v>https://doi.org/10.1021/acs.jctc.3c00527</x:v>
+        <x:v>https://doi.org/10.3390/s23125683</x:v>
       </x:c>
       <x:c r="F67" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3136,19 +3136,19 @@
     </x:row>
     <x:row r="68">
       <x:c r="A68" s="2" t="str">
-        <x:v>Programming Quantum Neural Networks on NISQ Systems: An Overview of Technologies and Methodologies</x:v>
+        <x:v>Optimization enabled Deep Quantum Neural Network for weed classification and density estimation</x:v>
       </x:c>
       <x:c r="B68" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C68" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D68" s="2" t="str">
-        <x:v>Stefano Markidis</x:v>
+        <x:v>Syamasudha Veeragandham, H. Santhi</x:v>
       </x:c>
       <x:c r="E68" s="2" t="str">
-        <x:v>https://doi.org/10.3390/e25040694</x:v>
+        <x:v>https://doi.org/10.1016/j.eswa.2023.122679</x:v>
       </x:c>
       <x:c r="F68" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3156,19 +3156,19 @@
     </x:row>
     <x:row r="69">
       <x:c r="A69" s="2" t="str">
-        <x:v>A duplication-free quantum neural network for universal approximation</x:v>
+        <x:v>Approximately Equivariant Quantum Neural Network for p4m Group Symmetries in Images</x:v>
       </x:c>
       <x:c r="B69" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C69" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
       </x:c>
       <x:c r="D69" s="2" t="str">
-        <x:v>Xiaokai Hou, Guanyu Zhou, Qingyu Li, Shan Jin, Xiaoting Wang</x:v>
+        <x:v>Su Yeon Chang, Michele Grossi, Bertrand Le Saux, Sofia Vallecorsa</x:v>
       </x:c>
       <x:c r="E69" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s11433-023-2098-8</x:v>
+        <x:v>https://doi.org/10.1109/QCE57702.2023.00033</x:v>
       </x:c>
       <x:c r="F69" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3176,7 +3176,7 @@
     </x:row>
     <x:row r="70">
       <x:c r="A70" s="2" t="str">
-        <x:v>Quantity study on a novel quantum neural network with alternately controlled gates for binary image classification</x:v>
+        <x:v>Estimating quantum mutual information through a quantum neural network</x:v>
       </x:c>
       <x:c r="B70" s="2" t="n">
         <x:v>2023</x:v>
@@ -3185,10 +3185,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D70" s="2" t="str">
-        <x:v>Qi Bai, Xianliang Hu</x:v>
+        <x:v>Myeongjin Shin, Junseo Lee &amp; Kabgyun Jeong</x:v>
       </x:c>
       <x:c r="E70" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s11128-023-03929-y</x:v>
+        <x:v>https://doi.org/10.1007/s11128-023-04253-1</x:v>
       </x:c>
       <x:c r="F70" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3196,19 +3196,19 @@
     </x:row>
     <x:row r="71">
       <x:c r="A71" s="2" t="str">
-        <x:v>Application of Quantum Neural Network for Solar Irradiance Forecasting: A Case Study Using the Folsom Dataset, California</x:v>
+        <x:v>Federated Quantum Neural Network With Quantum Teleportation for Resource Optimization in Future Wireless Communication</x:v>
       </x:c>
       <x:c r="B71" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C71" s="2" t="str">
-        <x:v>MDPI</x:v>
+        <x:v>IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
       </x:c>
       <x:c r="D71" s="2" t="str">
-        <x:v>Victor Oliveira Santos, Felipe Pinto Marinho, Paulo Alexandre Costa Rocha, Jesse Van Griensven Thé, Bahram Gharabaghi</x:v>
+        <x:v>Bhaskara Narottama, Soo Young Shin</x:v>
       </x:c>
       <x:c r="E71" s="2" t="str">
-        <x:v>https://doi.org/10.3390/en17143580</x:v>
+        <x:v>https://doi.org/10.1109/TVT.2023.3280459</x:v>
       </x:c>
       <x:c r="F71" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3216,19 +3216,19 @@
     </x:row>
     <x:row r="72">
       <x:c r="A72" s="2" t="str">
-        <x:v>Impact of barren plateaus countermeasures on the quantum neural network capacity to learn</x:v>
+        <x:v>Intrusion detection model using optimized quantum neural network and elliptical curve cryptography for data security</x:v>
       </x:c>
       <x:c r="B72" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C72" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>ScienceDirect</x:v>
       </x:c>
       <x:c r="D72" s="2" t="str">
-        <x:v>Jacob L. Cybulski, Thanh Nguyen</x:v>
+        <x:v>Heba Kadry, Ahmed Farouk, Elnomery A. Zanaty, Omar Reyad</x:v>
       </x:c>
       <x:c r="E72" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s11128-023-04187-8</x:v>
+        <x:v>https://doi.org/10.1016/j.aej.2023.03.072</x:v>
       </x:c>
       <x:c r="F72" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3236,19 +3236,19 @@
     </x:row>
     <x:row r="73">
       <x:c r="A73" s="2" t="str">
-        <x:v>Computing the gradients with respect to all parameters of a quantum neural network using a single circuit</x:v>
+        <x:v>Quantum Neural Network Inspired Hardware Adaptable Ansatz for Efficient Quantum Simulation of Chemical Systems</x:v>
       </x:c>
       <x:c r="B73" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C73" s="2" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>Chemical Theory and Computation</x:v>
       </x:c>
       <x:c r="D73" s="2" t="str">
-        <x:v>Guang Ping He</x:v>
+        <x:v>Xiongzhi Zeng, Yi FanJie Liu, Zhenyu Li, Jinlong Yang</x:v>
       </x:c>
       <x:c r="E73" s="2" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2307.08167</x:v>
+        <x:v>https://doi.org/10.1021/acs.jctc.3c00527</x:v>
       </x:c>
       <x:c r="F73" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3256,19 +3256,19 @@
     </x:row>
     <x:row r="74">
       <x:c r="A74" s="2" t="str">
-        <x:v>Universal Approximation Theorem and error bounds for quantum neural networks and quantum reservoirs</x:v>
+        <x:v>Programming Quantum Neural Networks on NISQ Systems: An Overview of Technologies and Methodologies</x:v>
       </x:c>
       <x:c r="B74" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C74" s="2" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D74" s="2" t="str">
-        <x:v>Lukas Gonon, Antoine Jacquier</x:v>
+        <x:v>Stefano Markidis</x:v>
       </x:c>
       <x:c r="E74" s="2" t="str">
-        <x:v>https://10.48550/arXiv.2307.12904</x:v>
+        <x:v>https://doi.org/10.3390/e25040694</x:v>
       </x:c>
       <x:c r="F74" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3276,19 +3276,19 @@
     </x:row>
     <x:row r="75">
       <x:c r="A75" s="2" t="str">
-        <x:v>Hybrid Classical-Quantum Neural Network for Improving Space Weather Detection and Early Warning Alerts</x:v>
+        <x:v>A duplication-free quantum neural network for universal approximation</x:v>
       </x:c>
       <x:c r="B75" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C75" s="2" t="str">
-        <x:v>IEEE</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D75" s="2" t="str">
-        <x:v>Ahmad Alomari, Sathish A. P. Kumar</x:v>
+        <x:v>Xiaokai Hou, Guanyu Zhou, Qingyu Li, Shan Jin, Xiaoting Wang</x:v>
       </x:c>
       <x:c r="E75" s="2" t="str">
-        <x:v>https://doi.org/10.1109/CCAAW57883.2023.10219316</x:v>
+        <x:v>https://doi.org/10.1007/s11433-023-2098-8</x:v>
       </x:c>
       <x:c r="F75" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3296,7 +3296,7 @@
     </x:row>
     <x:row r="76">
       <x:c r="A76" s="2" t="str">
-        <x:v>Hyperparameter importance and optimization of quantum neural networks across small datasets</x:v>
+        <x:v>Quantity study on a novel quantum neural network with alternately controlled gates for binary image classification</x:v>
       </x:c>
       <x:c r="B76" s="2" t="n">
         <x:v>2023</x:v>
@@ -3305,10 +3305,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D76" s="2" t="str">
-        <x:v>Charles Moussa, Yash J. Patel, Vedran Dunjko, Thomas Bäck, Jan N. van Rijn</x:v>
+        <x:v>Qi Bai, Xianliang Hu</x:v>
       </x:c>
       <x:c r="E76" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s10994-023-06389-8</x:v>
+        <x:v>https://doi.org/10.1007/s11128-023-03929-y</x:v>
       </x:c>
       <x:c r="F76" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3316,19 +3316,19 @@
     </x:row>
     <x:row r="77">
       <x:c r="A77" s="2" t="str">
-        <x:v>Quaternion Quantum Neural Network for Classification</x:v>
+        <x:v>Application of Quantum Neural Network for Solar Irradiance Forecasting: A Case Study Using the Folsom Dataset, California</x:v>
       </x:c>
       <x:c r="B77" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C77" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>MDPI</x:v>
       </x:c>
       <x:c r="D77" s="2" t="str">
-        <x:v>Guillermo Altamirano-Escobedo, Eduardo Bayro-Corrochano</x:v>
+        <x:v>Victor Oliveira Santos, Felipe Pinto Marinho, Paulo Alexandre Costa Rocha, Jesse Van Griensven Thé, Bahram Gharabaghi</x:v>
       </x:c>
       <x:c r="E77" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s00006-023-01280-0</x:v>
+        <x:v>https://doi.org/10.3390/en17143580</x:v>
       </x:c>
       <x:c r="F77" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3336,19 +3336,19 @@
     </x:row>
     <x:row r="78">
       <x:c r="A78" s="2" t="str">
-        <x:v>Variational Quantum Neural Networks (VQNNS) in Image Classification</x:v>
+        <x:v>Impact of barren plateaus countermeasures on the quantum neural network capacity to learn</x:v>
       </x:c>
       <x:c r="B78" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C78" s="2" t="str">
-        <x:v>arXiv</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D78" s="2" t="str">
-        <x:v>Meghashrita Das, Tirupati Bolisetti</x:v>
+        <x:v>Jacob L. Cybulski, Thanh Nguyen</x:v>
       </x:c>
       <x:c r="E78" s="2" t="str">
-        <x:v>https://doi.org/10.48550/arXiv.2303.05860</x:v>
+        <x:v>https://doi.org/10.1007/s11128-023-04187-8</x:v>
       </x:c>
       <x:c r="F78" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3356,19 +3356,19 @@
     </x:row>
     <x:row r="79">
       <x:c r="A79" s="2" t="str">
-        <x:v>Amplitude transformed quantum convolutional neural network</x:v>
+        <x:v>Computing the gradients with respect to all parameters of a quantum neural network using a single circuit</x:v>
       </x:c>
       <x:c r="B79" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C79" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D79" s="2" t="str">
-        <x:v>Shiqin Di, Jinchen Xu, Guoqiang Shu, Congcong Feng, Xiaodong Ding, Zheng Shan</x:v>
+        <x:v>Guang Ping He</x:v>
       </x:c>
       <x:c r="E79" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s10489-023-04581-w</x:v>
+        <x:v>https://doi.org/10.48550/arXiv.2307.08167</x:v>
       </x:c>
       <x:c r="F79" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3376,19 +3376,19 @@
     </x:row>
     <x:row r="80">
       <x:c r="A80" s="2" t="str">
-        <x:v>QTN-VQC: an end-to-end learning framework for quantum neural networks</x:v>
+        <x:v>Universal Approximation Theorem and error bounds for quantum neural networks and quantum reservoirs</x:v>
       </x:c>
       <x:c r="B80" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C80" s="2" t="str">
-        <x:v>IOPScience</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D80" s="2" t="str">
-        <x:v>Jun Qi, Chao-Han Yang, Pin-Yu Chen</x:v>
+        <x:v>Lukas Gonon, Antoine Jacquier</x:v>
       </x:c>
       <x:c r="E80" s="2" t="str">
-        <x:v>https://doi.org/10.1088/1402-4896/ad14d6</x:v>
+        <x:v>https://10.48550/arXiv.2307.12904</x:v>
       </x:c>
       <x:c r="F80" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3396,19 +3396,19 @@
     </x:row>
     <x:row r="81">
       <x:c r="A81" s="2" t="str">
-        <x:v>Resource saving via ensemble techniques for quantum neural networks</x:v>
+        <x:v>Hybrid Classical-Quantum Neural Network for Improving Space Weather Detection and Early Warning Alerts</x:v>
       </x:c>
       <x:c r="B81" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C81" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>IEEE</x:v>
       </x:c>
       <x:c r="D81" s="2" t="str">
-        <x:v>Massimiliano Incudini, Michele Grossi, Andrea Ceschini, Antonio Mandarino, Massimo Panella, Sofia Vallecorsa, David Windridge</x:v>
+        <x:v>Ahmad Alomari, Sathish A. P. Kumar</x:v>
       </x:c>
       <x:c r="E81" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00126-z</x:v>
+        <x:v>https://doi.org/10.1109/CCAAW57883.2023.10219316</x:v>
       </x:c>
       <x:c r="F81" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3416,7 +3416,7 @@
     </x:row>
     <x:row r="82">
       <x:c r="A82" s="2" t="str">
-        <x:v>Rapid training of quantum recurrent neural networks</x:v>
+        <x:v>Hyperparameter importance and optimization of quantum neural networks across small datasets</x:v>
       </x:c>
       <x:c r="B82" s="2" t="n">
         <x:v>2023</x:v>
@@ -3425,10 +3425,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D82" s="2" t="str">
-        <x:v>Michał Siemaszko, Adam Buraczewski, Bertrand Le Saux, Magdalena Stobińska </x:v>
+        <x:v>Charles Moussa, Yash J. Patel, Vedran Dunjko, Thomas Bäck, Jan N. van Rijn</x:v>
       </x:c>
       <x:c r="E82" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00117-0</x:v>
+        <x:v>https://doi.org/10.1007/s10994-023-06389-8</x:v>
       </x:c>
       <x:c r="F82" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3436,7 +3436,7 @@
     </x:row>
     <x:row r="83">
       <x:c r="A83" s="2" t="str">
-        <x:v>Linear-layer-enhanced quantum long short-term memory for carbon price forecasting</x:v>
+        <x:v>Quaternion Quantum Neural Network for Classification</x:v>
       </x:c>
       <x:c r="B83" s="2" t="n">
         <x:v>2023</x:v>
@@ -3445,10 +3445,10 @@
         <x:v>Springer</x:v>
       </x:c>
       <x:c r="D83" s="2" t="str">
-        <x:v>Yuji Cao, Xiyuan Zhou, Xiang Fei, Huan Zhao, Wenxuan Liu &amp; Junhua Zhao</x:v>
+        <x:v>Guillermo Altamirano-Escobedo, Eduardo Bayro-Corrochano</x:v>
       </x:c>
       <x:c r="E83" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00115-2</x:v>
+        <x:v>https://doi.org/10.1007/s00006-023-01280-0</x:v>
       </x:c>
       <x:c r="F83" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3456,19 +3456,19 @@
     </x:row>
     <x:row r="84">
       <x:c r="A84" s="2" t="str">
-        <x:v>An invitation to distributed quantum neural networks</x:v>
+        <x:v>Variational Quantum Neural Networks (VQNNS) in Image Classification</x:v>
       </x:c>
       <x:c r="B84" s="2" t="n">
         <x:v>2023</x:v>
       </x:c>
       <x:c r="C84" s="2" t="str">
-        <x:v>Springer</x:v>
+        <x:v>arXiv</x:v>
       </x:c>
       <x:c r="D84" s="2" t="str">
-        <x:v>Lirandë Pira &amp; Chris Ferrie </x:v>
+        <x:v>Meghashrita Das, Tirupati Bolisetti</x:v>
       </x:c>
       <x:c r="E84" s="2" t="str">
-        <x:v>https://doi.org/10.1007/s42484-023-00114-3</x:v>
+        <x:v>https://doi.org/10.48550/arXiv.2303.05860</x:v>
       </x:c>
       <x:c r="F84" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3476,19 +3476,19 @@
     </x:row>
     <x:row r="85">
       <x:c r="A85" s="2" t="str">
-        <x:v>Quantum Neural Network Compression</x:v>
+        <x:v>Amplitude transformed quantum convolutional neural network</x:v>
       </x:c>
       <x:c r="B85" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C85" s="2" t="str">
-        <x:v>Conference ICCAD</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D85" s="2" t="str">
-        <x:v>Zhirui Hu, Peiyan Dong, Zhepeng Wang, Youzuo Lin, Yanzhi Wang, Weiwen Jiang</x:v>
+        <x:v>Shiqin Di, Jinchen Xu, Guoqiang Shu, Congcong Feng, Xiaodong Ding, Zheng Shan</x:v>
       </x:c>
       <x:c r="E85" s="2" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3508352.3549382</x:v>
+        <x:v>https://doi.org/10.1007/s10489-023-04581-w</x:v>
       </x:c>
       <x:c r="F85" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3496,19 +3496,19 @@
     </x:row>
     <x:row r="86">
       <x:c r="A86" s="2" t="str">
-        <x:v>Quantum Neural Network Classifiers: A Tutorial</x:v>
+        <x:v>QTN-VQC: an end-to-end learning framework for quantum neural networks</x:v>
       </x:c>
       <x:c r="B86" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C86" s="2" t="str">
-        <x:v>SciPost Physics Lecture Notes</x:v>
+        <x:v>IOPScience</x:v>
       </x:c>
       <x:c r="D86" s="2" t="str">
-        <x:v>Weikang Li, Zhide Lu, Dong-Ling Deng</x:v>
+        <x:v>Jun Qi, Chao-Han Yang, Pin-Yu Chen</x:v>
       </x:c>
       <x:c r="E86" s="2" t="str">
-        <x:v>https://www.scipost.org/SciPostPhysLectNotes.61</x:v>
+        <x:v>https://doi.org/10.1088/1402-4896/ad14d6</x:v>
       </x:c>
       <x:c r="F86" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3516,19 +3516,19 @@
     </x:row>
     <x:row r="87">
       <x:c r="A87" s="2" t="str">
-        <x:v>Network attack detection scheme based on variational quantum neural network</x:v>
+        <x:v>Resource saving via ensemble techniques for quantum neural networks</x:v>
       </x:c>
       <x:c r="B87" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C87" s="2" t="str">
-        <x:v>The Journal of Supercomputing</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D87" s="2" t="str">
-        <x:v>Changqing Gong, Weiqi Guan, Abdullah Gani &amp; Han Qi</x:v>
+        <x:v>Massimiliano Incudini, Michele Grossi, Andrea Ceschini, Antonio Mandarino, Massimo Panella, Sofia Vallecorsa, David Windridge</x:v>
       </x:c>
       <x:c r="E87" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11227-022-04542-z</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00126-z</x:v>
       </x:c>
       <x:c r="F87" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3536,19 +3536,19 @@
     </x:row>
     <x:row r="88">
       <x:c r="A88" s="2" t="str">
-        <x:v>wpScalable Quantum Neural Networks for Classification</x:v>
+        <x:v>Rapid training of quantum recurrent neural networks</x:v>
       </x:c>
       <x:c r="B88" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C88" s="2" t="str">
-        <x:v>2022 IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D88" s="2" t="str">
-        <x:v>Jindi Wu; Zeyi Tao; Qun Li</x:v>
+        <x:v>Michał Siemaszko, Adam Buraczewski, Bertrand Le Saux, Magdalena Stobińska </x:v>
       </x:c>
       <x:c r="E88" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9951212</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00117-0</x:v>
       </x:c>
       <x:c r="F88" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3556,19 +3556,19 @@
     </x:row>
     <x:row r="89">
       <x:c r="A89" s="2" t="str">
-        <x:v>QuantumLeap: Hybrid quantum neural network for financial predictions</x:v>
+        <x:v>Linear-layer-enhanced quantum long short-term memory for carbon price forecasting</x:v>
       </x:c>
       <x:c r="B89" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C89" s="2" t="str">
-        <x:v>Elsevier</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D89" s="2" t="str">
-        <x:v>Eric Paquet, Farzan Soleymani</x:v>
+        <x:v>Yuji Cao, Xiyuan Zhou, Xiang Fei, Huan Zhao, Wenxuan Liu &amp; Junhua Zhao</x:v>
       </x:c>
       <x:c r="E89" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/pii/S0957417422000720</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00115-2</x:v>
       </x:c>
       <x:c r="F89" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3576,19 +3576,19 @@
     </x:row>
     <x:row r="90">
       <x:c r="A90" s="2" t="str">
-        <x:v>Quantum Robustness Verification: A Hybrid Quantum-Classical Neural Network Certification Algorithm</x:v>
+        <x:v>An invitation to distributed quantum neural networks</x:v>
       </x:c>
       <x:c r="B90" s="2" t="n">
-        <x:v>2022</x:v>
+        <x:v>2023</x:v>
       </x:c>
       <x:c r="C90" s="2" t="str">
-        <x:v>IEEE (Quantum Computing and Engineering (QCE))</x:v>
+        <x:v>Springer</x:v>
       </x:c>
       <x:c r="D90" s="2" t="str">
-        <x:v>Nicola Franco; Tom Wollschläger; Nicholas Gao; Jeanette Miriam Lorenz; Stephan Günnemann</x:v>
+        <x:v>Lirandë Pira &amp; Chris Ferrie </x:v>
       </x:c>
       <x:c r="E90" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9951230</x:v>
+        <x:v>https://doi.org/10.1007/s42484-023-00114-3</x:v>
       </x:c>
       <x:c r="F90" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3596,19 +3596,19 @@
     </x:row>
     <x:row r="91">
       <x:c r="A91" s="2" t="str">
-        <x:v>QNet: A Scalable and Noise-Resilient Quantum Neural Network Architecture for Noisy Intermediate-Scale Quantum Computers</x:v>
+        <x:v>Quantum Neural Network Compression</x:v>
       </x:c>
       <x:c r="B91" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C91" s="2" t="str">
-        <x:v>frontier</x:v>
+        <x:v>Conference ICCAD</x:v>
       </x:c>
       <x:c r="D91" s="2" t="str">
-        <x:v>Mahabubul Alam; Swaroop Ghosh</x:v>
+        <x:v>Zhirui Hu, Peiyan Dong, Zhepeng Wang, Youzuo Lin, Yanzhi Wang, Weiwen Jiang</x:v>
       </x:c>
       <x:c r="E91" s="2" t="str">
-        <x:v>https://www.frontiersin.org/journals/physics/articles/10.3389/fphy.2021.755139/full</x:v>
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3508352.3549382</x:v>
       </x:c>
       <x:c r="F91" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3616,19 +3616,19 @@
     </x:row>
     <x:row r="92">
       <x:c r="A92" s="2" t="str">
-        <x:v>Quantum neural network autoencoder and classifier applied to an industrial case study</x:v>
+        <x:v>Quantum Neural Network Classifiers: A Tutorial</x:v>
       </x:c>
       <x:c r="B92" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C92" s="2" t="str">
-        <x:v>SpringerLink</x:v>
+        <x:v>SciPost Physics Lecture Notes</x:v>
       </x:c>
       <x:c r="D92" s="2" t="str">
-        <x:v>    Stefano Mangini, Alessia Marruzzo, Marco Piantanida, Dario Gerace, Daniele Bajoni &amp; Chiara Macchiavello</x:v>
+        <x:v>Weikang Li, Zhide Lu, Dong-Ling Deng</x:v>
       </x:c>
       <x:c r="E92" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-022-00070-4</x:v>
+        <x:v>https://www.scipost.org/SciPostPhysLectNotes.61</x:v>
       </x:c>
       <x:c r="F92" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3636,19 +3636,19 @@
     </x:row>
     <x:row r="93">
       <x:c r="A93" s="2" t="str">
-        <x:v>QuClassi: A Hybrid Deep Neural Network Architecture based on Quantum State Fidelity</x:v>
+        <x:v>Network attack detection scheme based on variational quantum neural network</x:v>
       </x:c>
       <x:c r="B93" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C93" s="2" t="str">
-        <x:v>MLSys</x:v>
+        <x:v>The Journal of Supercomputing</x:v>
       </x:c>
       <x:c r="D93" s="2" t="str">
-        <x:v>Samuel A. Stein, Betis Baheri, Daniel Chen, Ying Mao, Qiang Guan, Ang Li, Shuai Xu, Caiwen Ding</x:v>
+        <x:v>Changqing Gong, Weiqi Guan, Abdullah Gani &amp; Han Qi</x:v>
       </x:c>
       <x:c r="E93" s="2" t="str">
-        <x:v>https://proceedings.mlsys.org/paper_files/paper/2022/hash/928f1160e52192e3e0017fb63ab65391-Abstract.html</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11227-022-04542-z</x:v>
       </x:c>
       <x:c r="F93" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3656,19 +3656,19 @@
     </x:row>
     <x:row r="94">
       <x:c r="A94" s="2" t="str">
-        <x:v>Trainability of Dissipative Perceptron-Based Quantum Neural Networks</x:v>
+        <x:v>wpScalable Quantum Neural Networks for Classification</x:v>
       </x:c>
       <x:c r="B94" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C94" s="2" t="str">
-        <x:v>Physical Review Letters</x:v>
+        <x:v>2022 IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
       </x:c>
       <x:c r="D94" s="2" t="str">
-        <x:v>Kunal Sharma, M. Cerezo, Lukasz Cincio, and Patrick J. Coles</x:v>
+        <x:v>Jindi Wu; Zeyi Tao; Qun Li</x:v>
       </x:c>
       <x:c r="E94" s="2" t="str">
-        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.128.180505</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9951212</x:v>
       </x:c>
       <x:c r="F94" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3676,19 +3676,19 @@
     </x:row>
     <x:row r="95">
       <x:c r="A95" s="2" t="str">
-        <x:v>Quantum neural networks</x:v>
+        <x:v>QuantumLeap: Hybrid quantum neural network for financial predictions</x:v>
       </x:c>
       <x:c r="B95" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C95" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D95" s="2" t="str">
-        <x:v>Kerstin Beer</x:v>
+        <x:v>Eric Paquet, Farzan Soleymani</x:v>
       </x:c>
       <x:c r="E95" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2205.08154</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/pii/S0957417422000720</x:v>
       </x:c>
       <x:c r="F95" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3696,19 +3696,19 @@
     </x:row>
     <x:row r="96">
       <x:c r="A96" s="2" t="str">
-        <x:v>The Dilemma of Quantum Neural Networks</x:v>
+        <x:v>Quantum Robustness Verification: A Hybrid Quantum-Classical Neural Network Certification Algorithm</x:v>
       </x:c>
       <x:c r="B96" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C96" s="2" t="str">
-        <x:v>IEEE Transactions on Neural Networks and Learning Systems</x:v>
+        <x:v>IEEE (Quantum Computing and Engineering (QCE))</x:v>
       </x:c>
       <x:c r="D96" s="2" t="str">
-        <x:v>Yang Qian; Xinbiao Wang; Yuxuan Du; Xingyao Wu; Dacheng Tao</x:v>
+        <x:v>Nicola Franco; Tom Wollschläger; Nicholas Gao; Jeanette Miriam Lorenz; Stephan Günnemann</x:v>
       </x:c>
       <x:c r="E96" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9908575</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9951230</x:v>
       </x:c>
       <x:c r="F96" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3716,19 +3716,19 @@
     </x:row>
     <x:row r="97">
       <x:c r="A97" s="2" t="str">
-        <x:v>Demonstrating Quantum Advantage in Hybrid Quantum Neural Networks for Model Capacity</x:v>
+        <x:v>QNet: A Scalable and Noise-Resilient Quantum Neural Network Architecture for Noisy Intermediate-Scale Quantum Computers</x:v>
       </x:c>
       <x:c r="B97" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C97" s="2" t="str">
-        <x:v>2022 IEEE International Conference on Rebooting Computing (ICRC)</x:v>
+        <x:v>frontier</x:v>
       </x:c>
       <x:c r="D97" s="2" t="str">
-        <x:v>Muhammad Kashif; Saif Al-Kuwari</x:v>
+        <x:v>Mahabubul Alam; Swaroop Ghosh</x:v>
       </x:c>
       <x:c r="E97" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/10062518</x:v>
+        <x:v>https://www.frontiersin.org/journals/physics/articles/10.3389/fphy.2021.755139/full</x:v>
       </x:c>
       <x:c r="F97" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3736,19 +3736,19 @@
     </x:row>
     <x:row r="98">
       <x:c r="A98" s="2" t="str">
-        <x:v>Variational algorithm of quantum neural network based on quantum particle swarm </x:v>
+        <x:v>Quantum neural network autoencoder and classifier applied to an industrial case study</x:v>
       </x:c>
       <x:c r="B98" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C98" s="2" t="str">
-        <x:v>Applied physics</x:v>
+        <x:v>SpringerLink</x:v>
       </x:c>
       <x:c r="D98" s="2" t="str">
-        <x:v>Yumin Dong; Jianshe Xie; Wanbin Hu; Cheng Liu; Yi Luo</x:v>
+        <x:v>    Stefano Mangini, Alessia Marruzzo, Marco Piantanida, Dario Gerace, Daniele Bajoni &amp; Chiara Macchiavello</x:v>
       </x:c>
       <x:c r="E98" s="2" t="str">
-        <x:v>https://pubs.aip.org/aip/jap/article-abstract/132/10/104401/2837384/Variational-algorithm-of-quantum-neural-network?redirectedFrom=fulltext</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s42484-022-00070-4</x:v>
       </x:c>
       <x:c r="F98" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3756,17 +3756,19 @@
     </x:row>
     <x:row r="99" s="2" customFormat="1">
       <x:c r="A99" s="2" t="str">
-        <x:v>Evaluation of Different Ansatze Designs for Quantum Neural Network Binary Classiers</x:v>
+        <x:v>QuClassi: A Hybrid Deep Neural Network Architecture based on Quantum State Fidelity</x:v>
       </x:c>
       <x:c r="B99" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="C99" s="2"/>
+      <x:c r="C99" s="2" t="str">
+        <x:v>MLSys</x:v>
+      </x:c>
       <x:c r="D99" s="2" t="str">
-        <x:v>Maha A. Metawei; Hazem Said; Hesham ElDeeb</x:v>
+        <x:v>Samuel A. Stein, Betis Baheri, Daniel Chen, Ying Mao, Qiang Guan, Ang Li, Shuai Xu, Caiwen Ding</x:v>
       </x:c>
       <x:c r="E99" s="2" t="str">
-        <x:v>https://doi.org/10.21203/rs.3.rs-1919180/v1</x:v>
+        <x:v>https://proceedings.mlsys.org/paper_files/paper/2022/hash/928f1160e52192e3e0017fb63ab65391-Abstract.html</x:v>
       </x:c>
       <x:c r="F99" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3774,19 +3776,19 @@
     </x:row>
     <x:row r="100" s="2" customFormat="1">
       <x:c r="A100" s="2" t="str">
-        <x:v>Binary Classification Quantum Neural Network Model Based on Optimized Grover Algorithm</x:v>
+        <x:v>Trainability of Dissipative Perceptron-Based Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B100" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C100" s="2" t="str">
-        <x:v>Mdpi</x:v>
+        <x:v>Physical Review Letters</x:v>
       </x:c>
       <x:c r="D100" s="2" t="str">
-        <x:v>by Wenlin Zhao, Yinuo Wang, Yingjie Qu, Hongyang Ma and Shumei Wang</x:v>
+        <x:v>Kunal Sharma, M. Cerezo, Lukasz Cincio, and Patrick J. Coles</x:v>
       </x:c>
       <x:c r="E100" s="2" t="str">
-        <x:v>https://www.mdpi.com/1099-4300/24/12/1783</x:v>
+        <x:v>https://journals.aps.org/prl/abstract/10.1103/PhysRevLett.128.180505</x:v>
       </x:c>
       <x:c r="F100" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3794,19 +3796,19 @@
     </x:row>
     <x:row r="101" s="2" customFormat="1">
       <x:c r="A101" s="2" t="str">
-        <x:v>Quantum Machine Learning Architecture for COVID-19 Classification Based on Synthetic Data Generation Using Conditional Adversarial Neural Network</x:v>
+        <x:v>Quantum neural networks</x:v>
       </x:c>
       <x:c r="B101" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C101" s="2" t="str">
-        <x:v>Cognitive Computation (Springer Link)</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D101" s="2" t="str">
-        <x:v>    Javaria Amin, Muhammad Sharif, Nadia Gul, Seifedine Kadry &amp; Chinmay Chakraborty</x:v>
+        <x:v>Kerstin Beer</x:v>
       </x:c>
       <x:c r="E101" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/S12559-021-09926-6</x:v>
+        <x:v>https://arxiv.org/abs/2205.08154</x:v>
       </x:c>
       <x:c r="F101" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3814,19 +3816,19 @@
     </x:row>
     <x:row r="102" s="2" customFormat="1">
       <x:c r="A102" s="2" t="str">
-        <x:v>A Multi-Classification Hybrid Quantum Neural Network Using an All-Qubit Multi-Observable Measurement Strategy</x:v>
+        <x:v>The Dilemma of Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B102" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C102" s="2" t="str">
-        <x:v>Mdpi</x:v>
+        <x:v>IEEE Transactions on Neural Networks and Learning Systems</x:v>
       </x:c>
       <x:c r="D102" s="2" t="str">
-        <x:v>Yi Zeng, Hao Wang, Jin He, Qijun Huang and Sheng Chang</x:v>
+        <x:v>Yang Qian; Xinbiao Wang; Yuxuan Du; Xingyao Wu; Dacheng Tao</x:v>
       </x:c>
       <x:c r="E102" s="2" t="str">
-        <x:v>https://www.mdpi.com/1099-4300/24/3/394</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9908575</x:v>
       </x:c>
       <x:c r="F102" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3834,19 +3836,19 @@
     </x:row>
     <x:row r="103" s="2" customFormat="1">
       <x:c r="A103" s="2" t="str">
-        <x:v>Automated Detection of Alzheimer’s via Hybrid Classical Quantum Neural Networks</x:v>
+        <x:v>Demonstrating Quantum Advantage in Hybrid Quantum Neural Networks for Model Capacity</x:v>
       </x:c>
       <x:c r="B103" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C103" s="2" t="str">
-        <x:v>Mdpi</x:v>
+        <x:v>2022 IEEE International Conference on Rebooting Computing (ICRC)</x:v>
       </x:c>
       <x:c r="D103" s="2" t="str">
-        <x:v>Tayyaba Shahwar, Junaid Zafar, Ahmad Almogren, Haroon Zafar, Ateeq Ur Rehman, Muhammad Shafiq and Habib Hamam</x:v>
+        <x:v>Muhammad Kashif; Saif Al-Kuwari</x:v>
       </x:c>
       <x:c r="E103" s="2" t="str">
-        <x:v>https://www.mdpi.com/2079-9292/11/5/721</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/10062518</x:v>
       </x:c>
       <x:c r="F103" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3854,19 +3856,19 @@
     </x:row>
     <x:row r="104" s="2" customFormat="1">
       <x:c r="A104" s="2" t="str">
-        <x:v>Creating Quantum Circuits for Training Perceptron Neural Networks on the Principles of Grover's Algorithm</x:v>
+        <x:v>Variational algorithm of quantum neural network based on quantum particle swarm </x:v>
       </x:c>
       <x:c r="B104" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C104" s="2" t="str">
-        <x:v>Systems of Signals Generating and Processing in the Field of on Board Communications (IEEE)</x:v>
+        <x:v>Applied physics</x:v>
       </x:c>
       <x:c r="D104" s="2" t="str">
-        <x:v>C. B. Pronin; O. I. Maksimychev; A. V. Ostroukh; A. V. Volosova; E. N. Matukhina</x:v>
+        <x:v>Yumin Dong; Jianshe Xie; Wanbin Hu; Cheng Liu; Yi Luo</x:v>
       </x:c>
       <x:c r="E104" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9744279</x:v>
+        <x:v>https://pubs.aip.org/aip/jap/article-abstract/132/10/104401/2837384/Variational-algorithm-of-quantum-neural-network?redirectedFrom=fulltext</x:v>
       </x:c>
       <x:c r="F104" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3874,19 +3876,17 @@
     </x:row>
     <x:row r="105" s="2" customFormat="1">
       <x:c r="A105" s="2" t="str">
-        <x:v>Symmetric Pruning in Quantum Neural Networks</x:v>
+        <x:v>Evaluation of Different Ansatze Designs for Quantum Neural Network Binary Classiers</x:v>
       </x:c>
       <x:c r="B105" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
-      <x:c r="C105" s="2" t="str">
-        <x:v>arxiv</x:v>
-      </x:c>
+      <x:c r="C105" s="2"/>
       <x:c r="D105" s="2" t="str">
-        <x:v>Xinbiao Wang, Junyu Liu, Tongliang Liu, Yong Luo, Yuxuan Du, Dacheng Tao</x:v>
+        <x:v>Maha A. Metawei; Hazem Said; Hesham ElDeeb</x:v>
       </x:c>
       <x:c r="E105" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2208.14057</x:v>
+        <x:v>https://doi.org/10.21203/rs.3.rs-1919180/v1</x:v>
       </x:c>
       <x:c r="F105" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3894,19 +3894,19 @@
     </x:row>
     <x:row r="106" s="2" customFormat="1">
       <x:c r="A106" s="2" t="str">
-        <x:v>Quantum Neural Networks and Topological Quantum Field Theories</x:v>
+        <x:v>Binary Classification Quantum Neural Network Model Based on Optimized Grover Algorithm</x:v>
       </x:c>
       <x:c r="B106" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C106" s="2" t="str">
-        <x:v>Elsevier</x:v>
+        <x:v>Mdpi</x:v>
       </x:c>
       <x:c r="D106" s="2" t="str">
-        <x:v>Antonino Marcianò a b, Deen Chen c, Filippo Fabrocini c d, Chris Fields e, Enrico Greco f, Niels Gresnigt g, Krid Jinklub c, Matteo Lulli h, Kostas Terzidis c, Emanuele Zappala</x:v>
+        <x:v>by Wenlin Zhao, Yinuo Wang, Yingjie Qu, Hongyang Ma and Shumei Wang</x:v>
       </x:c>
       <x:c r="E106" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0893608022002027</x:v>
+        <x:v>https://www.mdpi.com/1099-4300/24/12/1783</x:v>
       </x:c>
       <x:c r="F106" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3914,19 +3914,19 @@
     </x:row>
     <x:row r="107" s="2" customFormat="1">
       <x:c r="A107" s="2" t="str">
-        <x:v>An Evaluation of Hardware-Efficient Quantum Neural Networks for Image Data Classification</x:v>
+        <x:v>Quantum Machine Learning Architecture for COVID-19 Classification Based on Synthetic Data Generation Using Conditional Adversarial Neural Network</x:v>
       </x:c>
       <x:c r="B107" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C107" s="2" t="str">
-        <x:v>Mdpi</x:v>
+        <x:v>Cognitive Computation (Springer Link)</x:v>
       </x:c>
       <x:c r="D107" s="2" t="str">
-        <x:v>Tuyen Nguyen, Incheon Paik, Yutaka Watanobe and Truong Cong Thang</x:v>
+        <x:v>    Javaria Amin, Muhammad Sharif, Nadia Gul, Seifedine Kadry &amp; Chinmay Chakraborty</x:v>
       </x:c>
       <x:c r="E107" s="2" t="str">
-        <x:v>https://www.mdpi.com/2079-9292/11/3/437</x:v>
+        <x:v>https://link.springer.com/article/10.1007/S12559-021-09926-6</x:v>
       </x:c>
       <x:c r="F107" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3934,19 +3934,19 @@
     </x:row>
     <x:row r="108" s="2" customFormat="1">
       <x:c r="A108" s="2" t="str">
-        <x:v>Segmentation and classification of lymphoblastic leukaemia using quantum neural network</x:v>
+        <x:v>A Multi-Classification Hybrid Quantum Neural Network Using an All-Qubit Multi-Observable Measurement Strategy</x:v>
       </x:c>
       <x:c r="B108" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C108" s="2" t="str">
-        <x:v>Wiley</x:v>
+        <x:v>Mdpi</x:v>
       </x:c>
       <x:c r="D108" s="2" t="str">
-        <x:v>Javeria Amin, Muhammad Almas Anjum, Senka Krivic, Muhammad Irfan Sharif</x:v>
+        <x:v>Yi Zeng, Hao Wang, Jin He, Qijun Huang and Sheng Chang</x:v>
       </x:c>
       <x:c r="E108" s="2" t="str">
-        <x:v>https://onlinelibrary.wiley.com/doi/abs/10.1111/exsy.13225</x:v>
+        <x:v>https://www.mdpi.com/1099-4300/24/3/394</x:v>
       </x:c>
       <x:c r="F108" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3954,19 +3954,19 @@
     </x:row>
     <x:row r="109" s="2" customFormat="1">
       <x:c r="A109" s="2" t="str">
-        <x:v>Quantum Technology &amp; Quantum Neural Networks in Smart Grids Control: Premier Perspectives</x:v>
+        <x:v>Automated Detection of Alzheimer’s via Hybrid Classical Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B109" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C109" s="2" t="str">
-        <x:v>International Conference on Control, Instrumentation, and Automation (IEEE)</x:v>
+        <x:v>Mdpi</x:v>
       </x:c>
       <x:c r="D109" s="2" t="str">
-        <x:v>Ashkan Safari; Amir Aminzadeh Ghavifekr</x:v>
+        <x:v>Tayyaba Shahwar, Junaid Zafar, Ahmad Almogren, Haroon Zafar, Ateeq Ur Rehman, Muhammad Shafiq and Habib Hamam</x:v>
       </x:c>
       <x:c r="E109" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9737203</x:v>
+        <x:v>https://www.mdpi.com/2079-9292/11/5/721</x:v>
       </x:c>
       <x:c r="F109" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3974,19 +3974,19 @@
     </x:row>
     <x:row r="110" s="2" customFormat="1">
       <x:c r="A110" s="2" t="str">
-        <x:v>Superposition-enhanced quantum neural network for multi-class image classification</x:v>
+        <x:v>Creating Quantum Circuits for Training Perceptron Neural Networks on the Principles of Grover's Algorithm</x:v>
       </x:c>
       <x:c r="B110" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C110" s="2" t="str">
-        <x:v>Chinese Journal of Physics</x:v>
+        <x:v>Systems of Signals Generating and Processing in the Field of on Board Communications (IEEE)</x:v>
       </x:c>
       <x:c r="D110" s="2" t="str">
-        <x:v>Qi Bai, Xianliang Hu</x:v>
+        <x:v>C. B. Pronin; O. I. Maksimychev; A. V. Ostroukh; A. V. Volosova; E. N. Matukhina</x:v>
       </x:c>
       <x:c r="E110" s="2" t="str">
-        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0577907324001151</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9744279</x:v>
       </x:c>
       <x:c r="F110" s="2" t="str">
         <x:v>QNN</x:v>
@@ -3994,19 +3994,19 @@
     </x:row>
     <x:row r="111" s="2" customFormat="1">
       <x:c r="A111" s="2" t="str">
-        <x:v>Quantum-Inspired Neural Networks for Advanced AI Applications - A Scholarly Review of Quantum Computing Techniques in Neural Network Design</x:v>
+        <x:v>Symmetric Pruning in Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B111" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C111" s="2" t="str">
-        <x:v>Journal of Computational Intelligence and Robotics</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D111" s="2" t="str">
-        <x:v>Mohan Raparthi,  Venkata Siva Prakash Nimmagadda,  Mohit Kumar Sahu </x:v>
+        <x:v>Xinbiao Wang, Junyu Liu, Tongliang Liu, Yong Luo, Yuxuan Du, Dacheng Tao</x:v>
       </x:c>
       <x:c r="E111" s="2" t="str">
-        <x:v>https://thesciencebrigade.com/jcir/article/view/129</x:v>
+        <x:v>https://arxiv.org/abs/2208.14057</x:v>
       </x:c>
       <x:c r="F111" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4014,19 +4014,19 @@
     </x:row>
     <x:row r="112" s="2" customFormat="1">
       <x:c r="A112" s="2" t="str">
-        <x:v>Solving quantum master equations with deep quantum neural networks</x:v>
+        <x:v>Quantum Neural Networks and Topological Quantum Field Theories</x:v>
       </x:c>
       <x:c r="B112" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C112" s="2" t="str">
-        <x:v>Physical Review Research</x:v>
+        <x:v>Elsevier</x:v>
       </x:c>
       <x:c r="D112" s="2" t="str">
-        <x:v>Zidu Liu, L.-M. Duan, and Dong-Ling Deng</x:v>
+        <x:v>Antonino Marcianò a b, Deen Chen c, Filippo Fabrocini c d, Chris Fields e, Enrico Greco f, Niels Gresnigt g, Krid Jinklub c, Matteo Lulli h, Kostas Terzidis c, Emanuele Zappala</x:v>
       </x:c>
       <x:c r="E112" s="2" t="str">
-        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.013097</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0893608022002027</x:v>
       </x:c>
       <x:c r="F112" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4034,19 +4034,19 @@
     </x:row>
     <x:row r="113" s="2" customFormat="1">
       <x:c r="A113" s="2" t="str">
-        <x:v>Toward Physically Realizable Quantum Neural Networks</x:v>
+        <x:v>An Evaluation of Hardware-Efficient Quantum Neural Networks for Image Data Classification</x:v>
       </x:c>
       <x:c r="B113" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C113" s="2" t="str">
-        <x:v>AAAI Technical Track on Machine Learning</x:v>
+        <x:v>Mdpi</x:v>
       </x:c>
       <x:c r="D113" s="2" t="str">
-        <x:v>Mohsen Heidari, Ananth Grama, Wojciech Szpankowski </x:v>
+        <x:v>Tuyen Nguyen, Incheon Paik, Yutaka Watanobe and Truong Cong Thang</x:v>
       </x:c>
       <x:c r="E113" s="2" t="str">
-        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/20647</x:v>
+        <x:v>https://www.mdpi.com/2079-9292/11/3/437</x:v>
       </x:c>
       <x:c r="F113" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4054,19 +4054,19 @@
     </x:row>
     <x:row r="114" s="2" customFormat="1">
       <x:c r="A114" s="2" t="str">
-        <x:v>Face Patterns Analysis and Recognition System Based on Quantum Neural Network QNN</x:v>
+        <x:v>Segmentation and classification of lymphoblastic leukaemia using quantum neural network</x:v>
       </x:c>
       <x:c r="B114" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C114" s="2" t="str">
-        <x:v>International Journal of Interactive Mobile Technologies (iJIM)</x:v>
+        <x:v>Wiley</x:v>
       </x:c>
       <x:c r="D114" s="2" t="str">
-        <x:v>Haider TH. Salim Alrikabi, Ibtisam Aljazaery</x:v>
+        <x:v>Javeria Amin, Muhammad Almas Anjum, Senka Krivic, Muhammad Irfan Sharif</x:v>
       </x:c>
       <x:c r="E114" s="2" t="str">
-        <x:v>https://www.researchgate.net/profile/Abdul-Hadi-Alaidi/publication/364815012_Face_Patterns_Analysis_and_Recognition_System_Based_on_Quantum_Neural_Network_QNN/links/6375a16e54eb5f547cdbf731/Face-Patterns-Analysis-and-Recognition-System-Based-on-Quantum-Neural-Network-QNN.pdf</x:v>
+        <x:v>https://onlinelibrary.wiley.com/doi/abs/10.1111/exsy.13225</x:v>
       </x:c>
       <x:c r="F114" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4074,19 +4074,19 @@
     </x:row>
     <x:row r="115" s="2" customFormat="1">
       <x:c r="A115" s="2" t="str">
-        <x:v>Embedding Learning in Hybrid Quantum-Classical Neural Networks</x:v>
+        <x:v>Quantum Technology &amp; Quantum Neural Networks in Smart Grids Control: Premier Perspectives</x:v>
       </x:c>
       <x:c r="B115" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C115" s="2" t="str">
-        <x:v>2022 IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
+        <x:v>International Conference on Control, Instrumentation, and Automation (IEEE)</x:v>
       </x:c>
       <x:c r="D115" s="2" t="str">
-        <x:v>Minzhao Liu; Junyu Liu; Rui Liu; Henry Makhanov; Danylo Lykov; Anuj Apte</x:v>
+        <x:v>Ashkan Safari; Amir Aminzadeh Ghavifekr</x:v>
       </x:c>
       <x:c r="E115" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9951229</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9737203</x:v>
       </x:c>
       <x:c r="F115" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4094,19 +4094,19 @@
     </x:row>
     <x:row r="116" s="2" customFormat="1">
       <x:c r="A116" s="2" t="str">
-        <x:v>New quantum neural network designs</x:v>
+        <x:v>Superposition-enhanced quantum neural network for multi-class image classification</x:v>
       </x:c>
       <x:c r="B116" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C116" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Chinese Journal of Physics</x:v>
       </x:c>
       <x:c r="D116" s="2" t="str">
-        <x:v>Felix Petitzon</x:v>
+        <x:v>Qi Bai, Xianliang Hu</x:v>
       </x:c>
       <x:c r="E116" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2203.07872</x:v>
+        <x:v>https://www.sciencedirect.com/science/article/abs/pii/S0577907324001151</x:v>
       </x:c>
       <x:c r="F116" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4114,19 +4114,19 @@
     </x:row>
     <x:row r="117" s="2" customFormat="1">
       <x:c r="A117" s="2" t="str">
-        <x:v>Random Quantum Neural Networks (RQNN) for Noisy Image Recognition</x:v>
+        <x:v>Quantum-Inspired Neural Networks for Advanced AI Applications - A Scholarly Review of Quantum Computing Techniques in Neural Network Design</x:v>
       </x:c>
       <x:c r="B117" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C117" s="2" t="str">
-        <x:v>arxiv</x:v>
+        <x:v>Journal of Computational Intelligence and Robotics</x:v>
       </x:c>
       <x:c r="D117" s="2" t="str">
-        <x:v>Debanjan Konar, Erol Gelenbe, Soham Bhandary, Aditya Das Sarma, Attila Cangi</x:v>
+        <x:v>Mohan Raparthi,  Venkata Siva Prakash Nimmagadda,  Mohit Kumar Sahu </x:v>
       </x:c>
       <x:c r="E117" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2203.01764</x:v>
+        <x:v>https://thesciencebrigade.com/jcir/article/view/129</x:v>
       </x:c>
       <x:c r="F117" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4134,19 +4134,19 @@
     </x:row>
     <x:row r="118" s="2" customFormat="1">
       <x:c r="A118" s="2" t="str">
-        <x:v>Logarithmic Dimension Reduction for Quantum Neural Networks</x:v>
+        <x:v>Solving quantum master equations with deep quantum neural networks</x:v>
       </x:c>
       <x:c r="B118" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C118" s="2" t="str">
-        <x:v>Logarithmic Dimension Reduction for Quantum Neural Networks</x:v>
+        <x:v>Physical Review Research</x:v>
       </x:c>
       <x:c r="D118" s="2" t="str">
-        <x:v>Hankyul Baek, Soohyun Park, Joongheon Kim</x:v>
+        <x:v>Zidu Liu, L.-M. Duan, and Dong-Ling Deng</x:v>
       </x:c>
       <x:c r="E118" s="2" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3583780.3615240</x:v>
+        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.013097</x:v>
       </x:c>
       <x:c r="F118" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4154,19 +4154,19 @@
     </x:row>
     <x:row r="119" s="2" customFormat="1">
       <x:c r="A119" s="2" t="str">
-        <x:v>Bayesian Quantum Neural Networks</x:v>
+        <x:v>Toward Physically Realizable Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B119" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C119" s="2" t="str">
-        <x:v>IEEE Access</x:v>
+        <x:v>AAAI Technical Track on Machine Learning</x:v>
       </x:c>
       <x:c r="D119" s="2" t="str">
-        <x:v>Nam Nguyen; Kwang-Cheng Chen</x:v>
+        <x:v>Mohsen Heidari, Ananth Grama, Wojciech Szpankowski </x:v>
       </x:c>
       <x:c r="E119" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9759399</x:v>
+        <x:v>https://ojs.aaai.org/index.php/AAAI/article/view/20647</x:v>
       </x:c>
       <x:c r="F119" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4174,19 +4174,19 @@
     </x:row>
     <x:row r="120" s="2" customFormat="1">
       <x:c r="A120" s="2" t="str">
-        <x:v>Hyperparameter Importance of Quantum Neural Networks Across Small Datasets</x:v>
+        <x:v>Face Patterns Analysis and Recognition System Based on Quantum Neural Network QNN</x:v>
       </x:c>
       <x:c r="B120" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C120" s="2" t="str">
-        <x:v>Lecture Notes in Computer Science</x:v>
+        <x:v>International Journal of Interactive Mobile Technologies (iJIM)</x:v>
       </x:c>
       <x:c r="D120" s="2" t="str">
-        <x:v>    Charles Moussa, Jan N. van Rijn, Thomas Bäck &amp; Vedran Dunjko </x:v>
+        <x:v>Haider TH. Salim Alrikabi, Ibtisam Aljazaery</x:v>
       </x:c>
       <x:c r="E120" s="2" t="str">
-        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-18840-4_3</x:v>
+        <x:v>https://www.researchgate.net/profile/Abdul-Hadi-Alaidi/publication/364815012_Face_Patterns_Analysis_and_Recognition_System_Based_on_Quantum_Neural_Network_QNN/links/6375a16e54eb5f547cdbf731/Face-Patterns-Analysis-and-Recognition-System-Based-on-Quantum-Neural-Network-QNN.pdf</x:v>
       </x:c>
       <x:c r="F120" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4194,19 +4194,19 @@
     </x:row>
     <x:row r="121" s="2" customFormat="1">
       <x:c r="A121" s="2" t="str">
-        <x:v>Quantum neural networks force fields generation</x:v>
+        <x:v>Embedding Learning in Hybrid Quantum-Classical Neural Networks</x:v>
       </x:c>
       <x:c r="B121" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C121" s="2" t="str">
-        <x:v>Machine Learning: Science and Technology</x:v>
+        <x:v>2022 IEEE International Conference on Quantum Computing and Engineering (QCE)</x:v>
       </x:c>
       <x:c r="D121" s="2" t="str">
-        <x:v>Oriel Kiss, Francesco Tacchino4,1, Sofia Vallecorsa3 and Ivano Tavernelli</x:v>
+        <x:v>Minzhao Liu; Junyu Liu; Rui Liu; Henry Makhanov; Danylo Lykov; Anuj Apte</x:v>
       </x:c>
       <x:c r="E121" s="2" t="str">
-        <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ac7d3c/meta</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9951229</x:v>
       </x:c>
       <x:c r="F121" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4214,19 +4214,19 @@
     </x:row>
     <x:row r="122" s="2" customFormat="1">
       <x:c r="A122" s="2" t="str">
-        <x:v>Systematic improvement of neural network quantum states using Lanczos</x:v>
+        <x:v>New quantum neural network designs</x:v>
       </x:c>
       <x:c r="B122" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C122" s="2" t="str">
-        <x:v>Advances in Neural Information Processing Systems 35 (NeurIPS 2022)</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D122" s="2" t="str">
-        <x:v>Hongwei Chen, Douglas Hendry, Phillip Weinberg, Adrian Feiguin</x:v>
+        <x:v>Felix Petitzon</x:v>
       </x:c>
       <x:c r="E122" s="2" t="str">
-        <x:v>https://proceedings.neurips.cc/paper_files/paper/2022/hash/3173c427cb4ed2d5eaab029c17f221ae-Abstract-Conference.html</x:v>
+        <x:v>https://arxiv.org/abs/2203.07872</x:v>
       </x:c>
       <x:c r="F122" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4234,7 +4234,7 @@
     </x:row>
     <x:row r="123" s="2" customFormat="1">
       <x:c r="A123" s="2" t="str">
-        <x:v>A Hybrid Quantum-Classical Neural Network Architecture for Binary Classification</x:v>
+        <x:v>Random Quantum Neural Networks (RQNN) for Noisy Image Recognition</x:v>
       </x:c>
       <x:c r="B123" s="2" t="n">
         <x:v>2022</x:v>
@@ -4243,10 +4243,10 @@
         <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D123" s="2" t="str">
-        <x:v>Davis Arthur, Prasanna Date</x:v>
+        <x:v>Debanjan Konar, Erol Gelenbe, Soham Bhandary, Aditya Das Sarma, Attila Cangi</x:v>
       </x:c>
       <x:c r="E123" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2201.01820</x:v>
+        <x:v>https://arxiv.org/abs/2203.01764</x:v>
       </x:c>
       <x:c r="F123" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4254,19 +4254,19 @@
     </x:row>
     <x:row r="124" s="2" customFormat="1">
       <x:c r="A124" s="2" t="str">
-        <x:v>QuantumNAS: Noise-Adaptive Search for Robust Quantum Circuits</x:v>
+        <x:v>Logarithmic Dimension Reduction for Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B124" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C124" s="2" t="str">
-        <x:v>IEEE Symposium on High-Performance Computer Architecture</x:v>
+        <x:v>Logarithmic Dimension Reduction for Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="D124" s="2" t="str">
-        <x:v>Hanrui Wang; Yongshan Ding; Jiaqi Gu; Yujun Lin; David Z. Pan; Frederic T. Chong</x:v>
+        <x:v>Hankyul Baek, Soohyun Park, Joongheon Kim</x:v>
       </x:c>
       <x:c r="E124" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9773233</x:v>
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3583780.3615240</x:v>
       </x:c>
       <x:c r="F124" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4274,19 +4274,19 @@
     </x:row>
     <x:row r="125" s="2" customFormat="1">
       <x:c r="A125" s="2" t="str">
-        <x:v>Learnable antinoise-receiver algorithm based on a quantum feedforward neural network in optical quantum communication</x:v>
+        <x:v>Bayesian Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B125" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C125" s="2" t="str">
-        <x:v>covering atomic, molecular, and optical physics and quantum science</x:v>
+        <x:v>IEEE Access</x:v>
       </x:c>
       <x:c r="D125" s="2" t="str">
-        <x:v>Zhiguo Qu, Xinzhu Liu, and Le Sun</x:v>
+        <x:v>Nam Nguyen; Kwang-Cheng Chen</x:v>
       </x:c>
       <x:c r="E125" s="2" t="str">
-        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.052427</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9759399</x:v>
       </x:c>
       <x:c r="F125" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4294,19 +4294,19 @@
     </x:row>
     <x:row r="126" s="2" customFormat="1">
       <x:c r="A126" s="2" t="str">
-        <x:v>Quantum error reduction with deep neural network applied at the post-processing stage</x:v>
+        <x:v>Hyperparameter Importance of Quantum Neural Networks Across Small Datasets</x:v>
       </x:c>
       <x:c r="B126" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C126" s="2" t="str">
-        <x:v>Quantum Information Processing</x:v>
+        <x:v>Lecture Notes in Computer Science</x:v>
       </x:c>
       <x:c r="D126" s="2" t="str">
-        <x:v>Andrey Zhukov &amp; Walter Pogosov</x:v>
+        <x:v>    Charles Moussa, Jan N. van Rijn, Thomas Bäck &amp; Vedran Dunjko </x:v>
       </x:c>
       <x:c r="E126" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s11128-022-03433-9</x:v>
+        <x:v>https://link.springer.com/chapter/10.1007/978-3-031-18840-4_3</x:v>
       </x:c>
       <x:c r="F126" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4314,19 +4314,19 @@
     </x:row>
     <x:row r="127">
       <x:c r="A127" s="2" t="str">
-        <x:v>Learnability of Quantum Neural Networks</x:v>
+        <x:v>Quantum neural networks force fields generation</x:v>
       </x:c>
       <x:c r="B127" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C127" s="2" t="str">
-        <x:v>PRX QUANTUM 2</x:v>
+        <x:v>Machine Learning: Science and Technology</x:v>
       </x:c>
       <x:c r="D127" s="2" t="str">
-        <x:v>Yuxuan Du, Min-Hsiu Hsieh, Tongliang Liu, Shan You, and Dacheng Tao</x:v>
+        <x:v>Oriel Kiss, Francesco Tacchino4,1, Sofia Vallecorsa3 and Ivano Tavernelli</x:v>
       </x:c>
       <x:c r="E127" s="2" t="str">
-        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.3.030901</x:v>
+        <x:v>https://iopscience.iop.org/article/10.1088/2632-2153/ac7d3c/meta</x:v>
       </x:c>
       <x:c r="F127" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4334,19 +4334,19 @@
     </x:row>
     <x:row r="128">
       <x:c r="A128" s="2" t="str">
-        <x:v>Quantum phase detection generalization from marginal quantum neural network models</x:v>
+        <x:v>Systematic improvement of neural network quantum states using Lanczos</x:v>
       </x:c>
       <x:c r="B128" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C128" s="2" t="str">
-        <x:v>covering condensed matter and materials physics</x:v>
+        <x:v>Advances in Neural Information Processing Systems 35 (NeurIPS 2022)</x:v>
       </x:c>
       <x:c r="D128" s="2" t="str">
-        <x:v>Saverio Monaco, Oriel Kiss, Antonio Mandarino, Sofia Vallecorsa, and Michele Grossi</x:v>
+        <x:v>Hongwei Chen, Douglas Hendry, Phillip Weinberg, Adrian Feiguin</x:v>
       </x:c>
       <x:c r="E128" s="2" t="str">
-        <x:v>https://journals.aps.org/prb/abstract/10.1103/PhysRevB.107.L081105</x:v>
+        <x:v>https://proceedings.neurips.cc/paper_files/paper/2022/hash/3173c427cb4ed2d5eaab029c17f221ae-Abstract-Conference.html</x:v>
       </x:c>
       <x:c r="F128" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4354,7 +4354,7 @@
     </x:row>
     <x:row r="129">
       <x:c r="A129" s="2" t="str">
-        <x:v>Neural-Network Quantum States: A Systematic Review</x:v>
+        <x:v>A Hybrid Quantum-Classical Neural Network Architecture for Binary Classification</x:v>
       </x:c>
       <x:c r="B129" s="2" t="n">
         <x:v>2022</x:v>
@@ -4363,10 +4363,10 @@
         <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D129" s="2" t="str">
-        <x:v>David R. Vivas, Javier Madroñero, Victor Bucheli, Luis O. Gómez, John H. Reina</x:v>
+        <x:v>Davis Arthur, Prasanna Date</x:v>
       </x:c>
       <x:c r="E129" s="2" t="str">
-        <x:v>https://arxiv.org/abs/2204.12966</x:v>
+        <x:v>https://arxiv.org/abs/2201.01820</x:v>
       </x:c>
       <x:c r="F129" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4374,19 +4374,19 @@
     </x:row>
     <x:row r="130">
       <x:c r="A130" s="2" t="str">
-        <x:v>Neural-network quantum states for periodic systems in continuous space</x:v>
+        <x:v>QuantumNAS: Noise-Adaptive Search for Robust Quantum Circuits</x:v>
       </x:c>
       <x:c r="B130" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C130" s="2" t="str">
-        <x:v>Physical Review Research</x:v>
+        <x:v>IEEE Symposium on High-Performance Computer Architecture</x:v>
       </x:c>
       <x:c r="D130" s="2" t="str">
-        <x:v>Gabriel Pescia, Jiequn Han, Alessandro Lovato, Jianfeng Lu, and Giuseppe Carleo</x:v>
+        <x:v>Hanrui Wang; Yongshan Ding; Jiaqi Gu; Yujun Lin; David Z. Pan; Frederic T. Chong</x:v>
       </x:c>
       <x:c r="E130" s="2" t="str">
-        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.023138</x:v>
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9773233</x:v>
       </x:c>
       <x:c r="F130" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4394,19 +4394,19 @@
     </x:row>
     <x:row r="131">
       <x:c r="A131" s="2" t="str">
-        <x:v>Complex-valued Neural Network-based Quantum Language Models</x:v>
+        <x:v>Learnable antinoise-receiver algorithm based on a quantum feedforward neural network in optical quantum communication</x:v>
       </x:c>
       <x:c r="B131" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C131" s="2" t="str">
-        <x:v>ACM Transactions on Information Systems (TOIS)</x:v>
+        <x:v>covering atomic, molecular, and optical physics and quantum science</x:v>
       </x:c>
       <x:c r="D131" s="2" t="str">
-        <x:v>Peng Zhang, Wenjie Hui, Benyou Wang, Donghao Zhao, Dawei Song, Christina Lioma, Jakob Grue Simonsen</x:v>
+        <x:v>Zhiguo Qu, Xinzhu Liu, and Le Sun</x:v>
       </x:c>
       <x:c r="E131" s="2" t="str">
-        <x:v>https://dl.acm.org/doi/abs/10.1145/3505138</x:v>
+        <x:v>https://journals.aps.org/pra/abstract/10.1103/PhysRevA.105.052427</x:v>
       </x:c>
       <x:c r="F131" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4414,19 +4414,19 @@
     </x:row>
     <x:row r="132">
       <x:c r="A132" s="2" t="str">
-        <x:v>Exploring quantum perceptron and quantum neural network structures with a teacher-student scheme</x:v>
+        <x:v>Quantum error reduction with deep neural network applied at the post-processing stage</x:v>
       </x:c>
       <x:c r="B132" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C132" s="2" t="str">
-        <x:v>Quantum Machine Intelligence</x:v>
+        <x:v>Quantum Information Processing</x:v>
       </x:c>
       <x:c r="D132" s="2" t="str">
-        <x:v>Aikaterini Gratsea &amp; Patrick Huembeli</x:v>
+        <x:v>Andrey Zhukov &amp; Walter Pogosov</x:v>
       </x:c>
       <x:c r="E132" s="2" t="str">
-        <x:v>https://link.springer.com/article/10.1007/s42484-021-00058-6</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s11128-022-03433-9</x:v>
       </x:c>
       <x:c r="F132" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4434,19 +4434,19 @@
     </x:row>
     <x:row r="133">
       <x:c r="A133" s="2" t="str">
-        <x:v>Quantum Generative Adversarial Network and Quantum Neural Network for Image Classification</x:v>
+        <x:v>Learnability of Quantum Neural Networks</x:v>
       </x:c>
       <x:c r="B133" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C133" s="2" t="str">
-        <x:v>IEEE - Sustainable Computing and Data Communication Systems (ICSCDS)</x:v>
+        <x:v>PRX QUANTUM 2</x:v>
       </x:c>
       <x:c r="D133" s="2" t="str">
-        <x:v>Arun Pandian J; Kanchanadevi K; Vadem Chandu Mohan; Pulibandla Hari Krishna; Edagottu Govardhan</x:v>
+        <x:v>Yuxuan Du, Min-Hsiu Hsieh, Tongliang Liu, Shan You, and Dacheng Tao</x:v>
       </x:c>
       <x:c r="E133" s="2" t="str">
-        <x:v>https://ieeexplore.ieee.org/abstract/document/9760943</x:v>
+        <x:v>https://journals.aps.org/prxquantum/abstract/10.1103/PRXQuantum.3.030901</x:v>
       </x:c>
       <x:c r="F133" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4454,19 +4454,19 @@
     </x:row>
     <x:row r="134">
       <x:c r="A134" s="2" t="str">
-        <x:v>Parametric t-stochastic neighbor embedding with quantum neural network</x:v>
+        <x:v>Quantum phase detection generalization from marginal quantum neural network models</x:v>
       </x:c>
       <x:c r="B134" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C134" s="2" t="str">
-        <x:v>Physical Review Research</x:v>
+        <x:v>covering condensed matter and materials physics</x:v>
       </x:c>
       <x:c r="D134" s="2" t="str">
-        <x:v>Yoshiaki Kawase, Kosuke Mitarai, and Keisuke Fujii</x:v>
+        <x:v>Saverio Monaco, Oriel Kiss, Antonio Mandarino, Sofia Vallecorsa, and Michele Grossi</x:v>
       </x:c>
       <x:c r="E134" s="2" t="str">
-        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.043199</x:v>
+        <x:v>https://journals.aps.org/prb/abstract/10.1103/PhysRevB.107.L081105</x:v>
       </x:c>
       <x:c r="F134" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4474,19 +4474,19 @@
     </x:row>
     <x:row r="135">
       <x:c r="A135" s="2" t="str">
-        <x:v>Investigating Network Parameters in Neural-Network Quantum States</x:v>
+        <x:v>Neural-Network Quantum States: A Systematic Review</x:v>
       </x:c>
       <x:c r="B135" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C135" s="2" t="str">
-        <x:v>Physical Society of Japan</x:v>
+        <x:v>arxiv</x:v>
       </x:c>
       <x:c r="D135" s="2" t="str">
-        <x:v>Yusuke Nomura</x:v>
+        <x:v>David R. Vivas, Javier Madroñero, Victor Bucheli, Luis O. Gómez, John H. Reina</x:v>
       </x:c>
       <x:c r="E135" s="2" t="str">
-        <x:v>https://journals.jps.jp/doi/full/10.7566/JPSJ.91.054709</x:v>
+        <x:v>https://arxiv.org/abs/2204.12966</x:v>
       </x:c>
       <x:c r="F135" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4494,19 +4494,19 @@
     </x:row>
     <x:row r="136">
       <x:c r="A136" s="2" t="str">
-        <x:v>Quantum Neural Architecture Search with Quantum Circuits Metric and Bayesian Optimization</x:v>
+        <x:v>Neural-network quantum states for periodic systems in continuous space</x:v>
       </x:c>
       <x:c r="B136" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C136" s="2" t="str">
-        <x:v>ICML 2022 Workshop AI4Science</x:v>
+        <x:v>Physical Review Research</x:v>
       </x:c>
       <x:c r="D136" s="2" t="str">
-        <x:v>Trong Duong, Sang T. Truong, Minh Pham, Bao Bach, June-Koo Rhee</x:v>
+        <x:v>Gabriel Pescia, Jiequn Han, Alessandro Lovato, Jianfeng Lu, and Giuseppe Carleo</x:v>
       </x:c>
       <x:c r="E136" s="2" t="str">
-        <x:v>https://openreview.net/forum?id=n4_RjCTbS_2</x:v>
+        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.023138</x:v>
       </x:c>
       <x:c r="F136" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4514,19 +4514,19 @@
     </x:row>
     <x:row r="137">
       <x:c r="A137" s="2" t="str">
-        <x:v>Quantum Methods for Neural Networks and Application to Medical Image Classification</x:v>
+        <x:v>Complex-valued Neural Network-based Quantum Language Models</x:v>
       </x:c>
       <x:c r="B137" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C137" s="2" t="str">
-        <x:v>Quantum</x:v>
+        <x:v>ACM Transactions on Information Systems (TOIS)</x:v>
       </x:c>
       <x:c r="D137" s="2" t="str">
-        <x:v>Jonas Landman, Natansh Mathur, Yun Yvonna Li, Martin Strahm, Skander Kazdaghli, Anupam Prakash, and Iordanis Kerenidis</x:v>
+        <x:v>Peng Zhang, Wenjie Hui, Benyou Wang, Donghao Zhao, Dawei Song, Christina Lioma, Jakob Grue Simonsen</x:v>
       </x:c>
       <x:c r="E137" s="2" t="str">
-        <x:v>https://quantum-journal.org/papers/q-2022-12-22-881/</x:v>
+        <x:v>https://dl.acm.org/doi/abs/10.1145/3505138</x:v>
       </x:c>
       <x:c r="F137" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4534,19 +4534,19 @@
     </x:row>
     <x:row r="138">
       <x:c r="A138" s="2" t="str">
-        <x:v>Optical neural network quantum state tomography</x:v>
+        <x:v>Exploring quantum perceptron and quantum neural network structures with a teacher-student scheme</x:v>
       </x:c>
       <x:c r="B138" s="2" t="n">
         <x:v>2022</x:v>
       </x:c>
       <x:c r="C138" s="2" t="str">
-        <x:v>Advanced Photonics</x:v>
+        <x:v>Quantum Machine Intelligence</x:v>
       </x:c>
       <x:c r="D138" s="2" t="str">
-        <x:v>Ying Zuo, Chenfeng Cao, Ningping Cao, Xuanying Lai, Bei Zeng, Shengwang Du</x:v>
+        <x:v>Aikaterini Gratsea &amp; Patrick Huembeli</x:v>
       </x:c>
       <x:c r="E138" s="2" t="str">
-        <x:v>https://www.spiedigitallibrary.org/journals/advanced-photonics/volume-4/issue-2/026004/Optical-neural-network-quantum-state-tomography/10.1117/1.AP.4.2.026004.full</x:v>
+        <x:v>https://link.springer.com/article/10.1007/s42484-021-00058-6</x:v>
       </x:c>
       <x:c r="F138" s="2" t="str">
         <x:v>QNN</x:v>
@@ -4554,71 +4554,191 @@
     </x:row>
     <x:row r="139">
       <x:c r="A139" s="2" t="str">
+        <x:v>Quantum Generative Adversarial Network and Quantum Neural Network for Image Classification</x:v>
+      </x:c>
+      <x:c r="B139" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C139" s="2" t="str">
+        <x:v>IEEE - Sustainable Computing and Data Communication Systems (ICSCDS)</x:v>
+      </x:c>
+      <x:c r="D139" s="2" t="str">
+        <x:v>Arun Pandian J; Kanchanadevi K; Vadem Chandu Mohan; Pulibandla Hari Krishna; Edagottu Govardhan</x:v>
+      </x:c>
+      <x:c r="E139" s="2" t="str">
+        <x:v>https://ieeexplore.ieee.org/abstract/document/9760943</x:v>
+      </x:c>
+      <x:c r="F139" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="140">
+      <x:c r="A140" s="2" t="str">
+        <x:v>Parametric t-stochastic neighbor embedding with quantum neural network</x:v>
+      </x:c>
+      <x:c r="B140" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C140" s="2" t="str">
+        <x:v>Physical Review Research</x:v>
+      </x:c>
+      <x:c r="D140" s="2" t="str">
+        <x:v>Yoshiaki Kawase, Kosuke Mitarai, and Keisuke Fujii</x:v>
+      </x:c>
+      <x:c r="E140" s="2" t="str">
+        <x:v>https://journals.aps.org/prresearch/abstract/10.1103/PhysRevResearch.4.043199</x:v>
+      </x:c>
+      <x:c r="F140" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="141">
+      <x:c r="A141" s="2" t="str">
+        <x:v>Investigating Network Parameters in Neural-Network Quantum States</x:v>
+      </x:c>
+      <x:c r="B141" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C141" s="2" t="str">
+        <x:v>Physical Society of Japan</x:v>
+      </x:c>
+      <x:c r="D141" s="2" t="str">
+        <x:v>Yusuke Nomura</x:v>
+      </x:c>
+      <x:c r="E141" s="2" t="str">
+        <x:v>https://journals.jps.jp/doi/full/10.7566/JPSJ.91.054709</x:v>
+      </x:c>
+      <x:c r="F141" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="142">
+      <x:c r="A142" s="2" t="str">
+        <x:v>Quantum Neural Architecture Search with Quantum Circuits Metric and Bayesian Optimization</x:v>
+      </x:c>
+      <x:c r="B142" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C142" s="2" t="str">
+        <x:v>ICML 2022 Workshop AI4Science</x:v>
+      </x:c>
+      <x:c r="D142" s="2" t="str">
+        <x:v>Trong Duong, Sang T. Truong, Minh Pham, Bao Bach, June-Koo Rhee</x:v>
+      </x:c>
+      <x:c r="E142" s="2" t="str">
+        <x:v>https://openreview.net/forum?id=n4_RjCTbS_2</x:v>
+      </x:c>
+      <x:c r="F142" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="143">
+      <x:c r="A143" s="2" t="str">
+        <x:v>Quantum Methods for Neural Networks and Application to Medical Image Classification</x:v>
+      </x:c>
+      <x:c r="B143" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C143" s="2" t="str">
+        <x:v>Quantum</x:v>
+      </x:c>
+      <x:c r="D143" s="2" t="str">
+        <x:v>Jonas Landman, Natansh Mathur, Yun Yvonna Li, Martin Strahm, Skander Kazdaghli, Anupam Prakash, and Iordanis Kerenidis</x:v>
+      </x:c>
+      <x:c r="E143" s="2" t="str">
+        <x:v>https://quantum-journal.org/papers/q-2022-12-22-881/</x:v>
+      </x:c>
+      <x:c r="F143" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="144">
+      <x:c r="A144" s="2" t="str">
+        <x:v>Optical neural network quantum state tomography</x:v>
+      </x:c>
+      <x:c r="B144" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C144" s="2" t="str">
+        <x:v>Advanced Photonics</x:v>
+      </x:c>
+      <x:c r="D144" s="2" t="str">
+        <x:v>Ying Zuo, Chenfeng Cao, Ningping Cao, Xuanying Lai, Bei Zeng, Shengwang Du</x:v>
+      </x:c>
+      <x:c r="E144" s="2" t="str">
+        <x:v>https://www.spiedigitallibrary.org/journals/advanced-photonics/volume-4/issue-2/026004/Optical-neural-network-quantum-state-tomography/10.1117/1.AP.4.2.026004.full</x:v>
+      </x:c>
+      <x:c r="F144" s="2" t="str">
+        <x:v>QNN</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="145">
+      <x:c r="A145" s="2" t="str">
         <x:v>Negational symmetry of quantum neural networks for binary pattern classification</x:v>
       </x:c>
-      <x:c r="B139" s="2" t="n">
-        <x:v>2022</x:v>
-      </x:c>
-      <x:c r="C139" s="2" t="str">
+      <x:c r="B145" s="2" t="n">
+        <x:v>2022</x:v>
+      </x:c>
+      <x:c r="C145" s="2" t="str">
         <x:v>Pattern Recognition</x:v>
       </x:c>
-      <x:c r="D139" s="2" t="str">
+      <x:c r="D145" s="2" t="str">
         <x:v>Nanqing Dong , Michael Kampffmeyer , Irina Voiculescu , Eric Xing</x:v>
       </x:c>
-      <x:c r="E139" s="2" t="str">
+      <x:c r="E145" s="2" t="str">
         <x:v>https://www.sciencedirect.com/science/article/pii/S003132032200231X</x:v>
       </x:c>
-      <x:c r="F139" s="2" t="str">
+      <x:c r="F145" s="2" t="str">
         <x:v>QNN</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:hyperlinks>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="R7b2ecdfad48147ce"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R731aa8aac78541fd"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="R95c11df3b17a45a2"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R293c45e48ab54594"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="R6352687a80374c81"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="R93a566af80164f21"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="Rc2030adc3f404640"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R444bea7f9d044aec"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R6869efb289334415"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="Re554578a79a94ea0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="Rc5d8e43f529948cf"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R7224e448230443c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="Rb49842affd144727"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Rbf5a3056e12b4194"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="Rbc3267b4998041a7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R65253209717e4392"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="Rc2437a95dff44a34"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="Rdfa5a28829a5489e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="R7619a786debe4b1b"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R8229ebaf8ccb4277"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R806330b15c66433d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="R4d28a5b75fce47c6"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R21d15ef76d8f439e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="Rd5df346147d749b0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="Racc3997d0e2149d9"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="R0fa434febd964706"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="Ref54fab2dac34bd8"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R1f038740d6c44eb7"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="Rba1154d74c934090"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R3f2ecea6b0ba4868"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R21f1b067210a483c"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="R71e164a724f44c58"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="Rce1a7db0adbd4244"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R25bfaae3a15b41e5"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R5329013ed83242ba"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="R88ed5ec47028484e"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="Rb846f255789f4c0d"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="R41961476ee524b92"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="Rc412a29653c24cb0"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R46020320839f4671"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="R190c9a5ca3bf4ee3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="Rf2804cfdcf3c45b3"/>
-    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="R71da98a083124aa8"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E4" r:id="Rce840fced9da4203"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E5" r:id="R6609ca419b1940cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E7" r:id="Rf126c50859284b70"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E8" r:id="R3f2048d1c0514c66"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E21" r:id="Refe061018d514fee"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E22" r:id="Rf290af7390d345c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E23" r:id="R7439476ab88d477b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E26" r:id="R2abd428a99f44fcb"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E34" r:id="R02ce0a28e3d54e16"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E39" r:id="Rb0bafbe30d7f43e7"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E40" r:id="R4d8ee17e7af748a5"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E41" r:id="R364884efa9a84b19"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E43" r:id="R31a725c8e9e3492b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E44" r:id="Rcea9a847af00496e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E45" r:id="Raeb8dd0ff030480a"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E46" r:id="R22bb60385bcc4102"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E47" r:id="R9d9754d282934b27"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E48" r:id="Rd063249ba8ce4868"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E49" r:id="Raf66bcd8c2a54440"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E50" r:id="R39b422e4eef64600"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E51" r:id="R52defdbe750046c9"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E52" r:id="Ra23b0814e70e49cc"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E53" r:id="R2af0d51435644052"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E54" r:id="Rdb08cdadfe744276"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E55" r:id="Rea063aca7be744ff"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E56" r:id="Rc7b2dcd8058a4134"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E57" r:id="R2b9086eb73f644c6"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E58" r:id="R85158a05f0b3418c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E59" r:id="R80060cdb117c4768"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E60" r:id="R089e2769be584730"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E61" r:id="R1c10065451fe42aa"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E62" r:id="R94141c007762495e"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E63" r:id="R097bab76a87a4734"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E64" r:id="R36ee8b20b73c45cf"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E65" r:id="R9e218e929b174750"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E66" r:id="Ra361129e42d24a37"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E67" r:id="Rfca6ba1e0c2444c0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E68" r:id="R568ec824bdb94599"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E69" r:id="Ra9bff2546b81474c"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E70" r:id="R3e821372b075489f"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E71" r:id="R38086c6e9422499b"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E72" r:id="R77d659629e7445b0"/>
+    <x:hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="E85" r:id="R7a7e878a89b7441a"/>
   </x:hyperlinks>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R5de46d6870cd45a3"/>
+  <x:drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbe8b05715e4c47d2"/>
 </x:worksheet>
 </file>
</xml_diff>